<commit_message>
fix: Removed background shading for Cambio de guardia rows in Excel export
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -1858,112 +1858,112 @@
       <c r="V15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>03208053</t>
         </is>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>MORETO BERMEO</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>FRANCO</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="5" t="inlineStr">
         <is>
           <t>Mantenimiento</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G16" s="12" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I16" s="12" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J16" s="12" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>06:32</t>
         </is>
       </c>
-      <c r="K16" s="12" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L16" s="12" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>17:23</t>
         </is>
       </c>
-      <c r="M16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P16" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" s="12" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O16" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q16" s="6" t="inlineStr">
         <is>
           <t>10:23</t>
         </is>
       </c>
-      <c r="R16" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S16" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T16" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U16" s="12" t="inlineStr">
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S16" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T16" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U16" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V16" s="11" t="inlineStr"/>
+      <c r="V16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -3718,112 +3718,112 @@
       <c r="V32" s="5" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>42626422</t>
         </is>
       </c>
-      <c r="B33" s="11" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>ALVARADO BERMEO</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>NEPTALI</t>
         </is>
       </c>
-      <c r="D33" s="11" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E33" s="11" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F33" s="12" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G33" s="12" t="inlineStr">
+      <c r="G33" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H33" s="12" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I33" s="12" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J33" s="12" t="inlineStr">
+      <c r="J33" s="6" t="inlineStr">
         <is>
           <t>04:45</t>
         </is>
       </c>
-      <c r="K33" s="12" t="inlineStr">
+      <c r="K33" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L33" s="12" t="inlineStr">
+      <c r="L33" s="6" t="inlineStr">
         <is>
           <t>16:52</t>
         </is>
       </c>
-      <c r="M33" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N33" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O33" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P33" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q33" s="12" t="inlineStr">
+      <c r="M33" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N33" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O33" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P33" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q33" s="6" t="inlineStr">
         <is>
           <t>11:53</t>
         </is>
       </c>
-      <c r="R33" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S33" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T33" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U33" s="12" t="inlineStr">
+      <c r="R33" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S33" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T33" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U33" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V33" s="11" t="inlineStr"/>
+      <c r="V33" s="5" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -5138,112 +5138,112 @@
       <c r="V45" s="5" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="10" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>45119078</t>
         </is>
       </c>
-      <c r="B46" s="11" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>CURINAMBE SANCHEZ</t>
         </is>
       </c>
-      <c r="C46" s="11" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr">
         <is>
           <t>JOSELITO</t>
         </is>
       </c>
-      <c r="D46" s="11" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E46" s="11" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F46" s="12" t="inlineStr">
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G46" s="12" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H46" s="12" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I46" s="12" t="inlineStr">
+      <c r="I46" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J46" s="12" t="inlineStr">
+      <c r="J46" s="6" t="inlineStr">
         <is>
           <t>04:49</t>
         </is>
       </c>
-      <c r="K46" s="12" t="inlineStr">
+      <c r="K46" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L46" s="12" t="inlineStr">
+      <c r="L46" s="6" t="inlineStr">
         <is>
           <t>16:53</t>
         </is>
       </c>
-      <c r="M46" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N46" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O46" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P46" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q46" s="12" t="inlineStr">
+      <c r="M46" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N46" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O46" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P46" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q46" s="6" t="inlineStr">
         <is>
           <t>11:53</t>
         </is>
       </c>
-      <c r="R46" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S46" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T46" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U46" s="12" t="inlineStr">
+      <c r="R46" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S46" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T46" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U46" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V46" s="11" t="inlineStr"/>
+      <c r="V46" s="5" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -6434,112 +6434,112 @@
       <c r="V57" s="5" t="inlineStr"/>
     </row>
     <row r="58" ht="20" customHeight="1">
-      <c r="A58" s="10" t="inlineStr">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>47591578</t>
         </is>
       </c>
-      <c r="B58" s="11" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr">
         <is>
           <t>NINAQUISPE JACOBO</t>
         </is>
       </c>
-      <c r="C58" s="11" t="inlineStr">
+      <c r="C58" s="5" t="inlineStr">
         <is>
           <t>LUIS MIGUEL</t>
         </is>
       </c>
-      <c r="D58" s="11" t="inlineStr">
+      <c r="D58" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E58" s="11" t="inlineStr">
+      <c r="E58" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F58" s="12" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G58" s="12" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H58" s="12" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I58" s="12" t="inlineStr">
+      <c r="I58" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J58" s="12" t="inlineStr">
+      <c r="J58" s="6" t="inlineStr">
         <is>
           <t>04:55</t>
         </is>
       </c>
-      <c r="K58" s="12" t="inlineStr">
+      <c r="K58" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L58" s="12" t="inlineStr">
+      <c r="L58" s="6" t="inlineStr">
         <is>
           <t>16:53</t>
         </is>
       </c>
-      <c r="M58" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N58" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O58" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P58" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q58" s="12" t="inlineStr">
+      <c r="M58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P58" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q58" s="6" t="inlineStr">
         <is>
           <t>11:53</t>
         </is>
       </c>
-      <c r="R58" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S58" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T58" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U58" s="12" t="inlineStr">
+      <c r="R58" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S58" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T58" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U58" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V58" s="11" t="inlineStr"/>
+      <c r="V58" s="5" t="inlineStr"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -8294,220 +8294,220 @@
       <c r="V74" s="5" t="inlineStr"/>
     </row>
     <row r="75" ht="20" customHeight="1">
-      <c r="A75" s="10" t="inlineStr">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>48790853</t>
         </is>
       </c>
-      <c r="B75" s="11" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>GUERRA SAJAMI</t>
         </is>
       </c>
-      <c r="C75" s="11" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>SANGABIL</t>
         </is>
       </c>
-      <c r="D75" s="11" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E75" s="11" t="inlineStr">
+      <c r="E75" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F75" s="12" t="inlineStr">
+      <c r="F75" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G75" s="12" t="inlineStr">
+      <c r="G75" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H75" s="12" t="inlineStr">
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I75" s="12" t="inlineStr">
+      <c r="I75" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J75" s="12" t="inlineStr">
+      <c r="J75" s="6" t="inlineStr">
         <is>
           <t>18:40</t>
         </is>
       </c>
-      <c r="K75" s="12" t="inlineStr">
+      <c r="K75" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L75" s="12" t="inlineStr">
+      <c r="L75" s="6" t="inlineStr">
         <is>
           <t>05:00</t>
         </is>
       </c>
-      <c r="M75" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N75" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O75" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P75" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q75" s="12" t="inlineStr">
+      <c r="M75" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N75" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O75" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P75" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q75" s="6" t="inlineStr">
         <is>
           <t>10:01</t>
         </is>
       </c>
-      <c r="R75" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S75" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T75" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U75" s="12" t="inlineStr">
+      <c r="R75" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S75" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T75" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U75" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V75" s="11" t="inlineStr"/>
+      <c r="V75" s="5" t="inlineStr"/>
     </row>
     <row r="76" ht="20" customHeight="1">
-      <c r="A76" s="10" t="inlineStr">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>48790853</t>
         </is>
       </c>
-      <c r="B76" s="11" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>GUERRA SAJAMI</t>
         </is>
       </c>
-      <c r="C76" s="11" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr">
         <is>
           <t>SANGABIL</t>
         </is>
       </c>
-      <c r="D76" s="11" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E76" s="11" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F76" s="12" t="inlineStr">
+      <c r="F76" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G76" s="12" t="inlineStr">
+      <c r="G76" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H76" s="12" t="inlineStr">
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I76" s="12" t="inlineStr">
+      <c r="I76" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J76" s="12" t="inlineStr">
+      <c r="J76" s="6" t="inlineStr">
         <is>
           <t>16:49</t>
         </is>
       </c>
-      <c r="K76" s="12" t="inlineStr">
+      <c r="K76" s="6" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="L76" s="12" t="inlineStr">
+      <c r="L76" s="6" t="inlineStr">
         <is>
           <t>07:09</t>
         </is>
       </c>
-      <c r="M76" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N76" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O76" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P76" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q76" s="12" t="inlineStr">
+      <c r="M76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P76" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q76" s="6" t="inlineStr">
         <is>
           <t>14:10</t>
         </is>
       </c>
-      <c r="R76" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S76" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T76" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U76" s="12" t="inlineStr">
+      <c r="R76" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S76" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T76" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U76" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V76" s="11" t="inlineStr"/>
+      <c r="V76" s="5" t="inlineStr"/>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
@@ -10590,220 +10590,220 @@
       </c>
     </row>
     <row r="96" ht="20" customHeight="1">
-      <c r="A96" s="10" t="inlineStr">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>70088280</t>
         </is>
       </c>
-      <c r="B96" s="11" t="inlineStr">
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>RAMIREZ GUERRERO</t>
         </is>
       </c>
-      <c r="C96" s="11" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>LUIS FERNANDO</t>
         </is>
       </c>
-      <c r="D96" s="11" t="inlineStr">
+      <c r="D96" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E96" s="11" t="inlineStr">
+      <c r="E96" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F96" s="12" t="inlineStr">
+      <c r="F96" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G96" s="12" t="inlineStr">
+      <c r="G96" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H96" s="12" t="inlineStr">
+      <c r="H96" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I96" s="12" t="inlineStr">
+      <c r="I96" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J96" s="12" t="inlineStr">
+      <c r="J96" s="6" t="inlineStr">
         <is>
           <t>18:31</t>
         </is>
       </c>
-      <c r="K96" s="12" t="inlineStr">
+      <c r="K96" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L96" s="12" t="inlineStr">
+      <c r="L96" s="6" t="inlineStr">
         <is>
           <t>04:58</t>
         </is>
       </c>
-      <c r="M96" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N96" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O96" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P96" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q96" s="12" t="inlineStr">
+      <c r="M96" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N96" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O96" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P96" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q96" s="6" t="inlineStr">
         <is>
           <t>09:58</t>
         </is>
       </c>
-      <c r="R96" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S96" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T96" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U96" s="12" t="inlineStr">
+      <c r="R96" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S96" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T96" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U96" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V96" s="11" t="inlineStr"/>
+      <c r="V96" s="5" t="inlineStr"/>
     </row>
     <row r="97" ht="20" customHeight="1">
-      <c r="A97" s="10" t="inlineStr">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>70088280</t>
         </is>
       </c>
-      <c r="B97" s="11" t="inlineStr">
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>RAMIREZ GUERRERO</t>
         </is>
       </c>
-      <c r="C97" s="11" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>LUIS FERNANDO</t>
         </is>
       </c>
-      <c r="D97" s="11" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E97" s="11" t="inlineStr">
+      <c r="E97" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F97" s="12" t="inlineStr">
+      <c r="F97" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G97" s="12" t="inlineStr">
+      <c r="G97" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H97" s="12" t="inlineStr">
+      <c r="H97" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I97" s="12" t="inlineStr">
+      <c r="I97" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J97" s="12" t="inlineStr">
+      <c r="J97" s="6" t="inlineStr">
         <is>
           <t>16:33</t>
         </is>
       </c>
-      <c r="K97" s="12" t="inlineStr">
+      <c r="K97" s="6" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="L97" s="12" t="inlineStr">
+      <c r="L97" s="6" t="inlineStr">
         <is>
           <t>07:04</t>
         </is>
       </c>
-      <c r="M97" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N97" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O97" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P97" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q97" s="12" t="inlineStr">
+      <c r="M97" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N97" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O97" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P97" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q97" s="6" t="inlineStr">
         <is>
           <t>14:04</t>
         </is>
       </c>
-      <c r="R97" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S97" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T97" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U97" s="12" t="inlineStr">
+      <c r="R97" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S97" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T97" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U97" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V97" s="11" t="inlineStr"/>
+      <c r="V97" s="5" t="inlineStr"/>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="10" t="inlineStr">
@@ -12762,220 +12762,220 @@
       <c r="V115" s="5" t="inlineStr"/>
     </row>
     <row r="116" ht="20" customHeight="1">
-      <c r="A116" s="10" t="inlineStr">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>71710169</t>
         </is>
       </c>
-      <c r="B116" s="11" t="inlineStr">
+      <c r="B116" s="5" t="inlineStr">
         <is>
           <t>INFANTES FERNANDEZ</t>
         </is>
       </c>
-      <c r="C116" s="11" t="inlineStr">
+      <c r="C116" s="5" t="inlineStr">
         <is>
           <t>MICHAEL JUNIOR</t>
         </is>
       </c>
-      <c r="D116" s="11" t="inlineStr">
+      <c r="D116" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E116" s="11" t="inlineStr">
+      <c r="E116" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F116" s="12" t="inlineStr">
+      <c r="F116" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G116" s="12" t="inlineStr">
+      <c r="G116" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H116" s="12" t="inlineStr">
+      <c r="H116" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I116" s="12" t="inlineStr">
+      <c r="I116" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J116" s="12" t="inlineStr">
+      <c r="J116" s="6" t="inlineStr">
         <is>
           <t>18:29</t>
         </is>
       </c>
-      <c r="K116" s="12" t="inlineStr">
+      <c r="K116" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L116" s="12" t="inlineStr">
+      <c r="L116" s="6" t="inlineStr">
         <is>
           <t>04:56</t>
         </is>
       </c>
-      <c r="M116" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N116" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O116" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P116" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q116" s="12" t="inlineStr">
+      <c r="M116" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N116" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O116" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P116" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q116" s="6" t="inlineStr">
         <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="R116" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S116" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T116" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U116" s="12" t="inlineStr">
+      <c r="R116" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S116" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T116" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U116" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V116" s="11" t="inlineStr"/>
+      <c r="V116" s="5" t="inlineStr"/>
     </row>
     <row r="117" ht="20" customHeight="1">
-      <c r="A117" s="10" t="inlineStr">
+      <c r="A117" s="4" t="inlineStr">
         <is>
           <t>71710169</t>
         </is>
       </c>
-      <c r="B117" s="11" t="inlineStr">
+      <c r="B117" s="5" t="inlineStr">
         <is>
           <t>INFANTES FERNANDEZ</t>
         </is>
       </c>
-      <c r="C117" s="11" t="inlineStr">
+      <c r="C117" s="5" t="inlineStr">
         <is>
           <t>MICHAEL JUNIOR</t>
         </is>
       </c>
-      <c r="D117" s="11" t="inlineStr">
+      <c r="D117" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E117" s="11" t="inlineStr">
+      <c r="E117" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F117" s="12" t="inlineStr">
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G117" s="12" t="inlineStr">
+      <c r="G117" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H117" s="12" t="inlineStr">
+      <c r="H117" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I117" s="12" t="inlineStr">
+      <c r="I117" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J117" s="12" t="inlineStr">
+      <c r="J117" s="6" t="inlineStr">
         <is>
           <t>16:57</t>
         </is>
       </c>
-      <c r="K117" s="12" t="inlineStr">
+      <c r="K117" s="6" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="L117" s="12" t="inlineStr">
+      <c r="L117" s="6" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="M117" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N117" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O117" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P117" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q117" s="12" t="inlineStr">
+      <c r="M117" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N117" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O117" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P117" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q117" s="6" t="inlineStr">
         <is>
           <t>14:01</t>
         </is>
       </c>
-      <c r="R117" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S117" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T117" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U117" s="12" t="inlineStr">
+      <c r="R117" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S117" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T117" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U117" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V117" s="11" t="inlineStr"/>
+      <c r="V117" s="5" t="inlineStr"/>
     </row>
     <row r="118" ht="20" customHeight="1">
       <c r="A118" s="10" t="inlineStr">
@@ -13306,220 +13306,220 @@
       <c r="V120" s="5" t="inlineStr"/>
     </row>
     <row r="121" ht="20" customHeight="1">
-      <c r="A121" s="10" t="inlineStr">
+      <c r="A121" s="4" t="inlineStr">
         <is>
           <t>71710175</t>
         </is>
       </c>
-      <c r="B121" s="11" t="inlineStr">
+      <c r="B121" s="5" t="inlineStr">
         <is>
           <t>INFANTES FERNANDEZ</t>
         </is>
       </c>
-      <c r="C121" s="11" t="inlineStr">
+      <c r="C121" s="5" t="inlineStr">
         <is>
           <t>BRANDOM VALDEMAR</t>
         </is>
       </c>
-      <c r="D121" s="11" t="inlineStr">
+      <c r="D121" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E121" s="11" t="inlineStr">
+      <c r="E121" s="5" t="inlineStr">
         <is>
           <t>Maquinaria Pesada</t>
         </is>
       </c>
-      <c r="F121" s="12" t="inlineStr">
+      <c r="F121" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G121" s="12" t="inlineStr">
+      <c r="G121" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H121" s="12" t="inlineStr">
+      <c r="H121" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I121" s="12" t="inlineStr">
+      <c r="I121" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J121" s="12" t="inlineStr">
+      <c r="J121" s="6" t="inlineStr">
         <is>
           <t>18:29</t>
         </is>
       </c>
-      <c r="K121" s="12" t="inlineStr">
+      <c r="K121" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L121" s="12" t="inlineStr">
+      <c r="L121" s="6" t="inlineStr">
         <is>
           <t>05:01</t>
         </is>
       </c>
-      <c r="M121" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N121" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O121" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P121" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q121" s="12" t="inlineStr">
+      <c r="M121" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N121" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O121" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P121" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q121" s="6" t="inlineStr">
         <is>
           <t>10:01</t>
         </is>
       </c>
-      <c r="R121" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S121" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T121" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U121" s="12" t="inlineStr">
+      <c r="R121" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S121" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T121" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U121" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V121" s="11" t="inlineStr"/>
+      <c r="V121" s="5" t="inlineStr"/>
     </row>
     <row r="122" ht="20" customHeight="1">
-      <c r="A122" s="10" t="inlineStr">
+      <c r="A122" s="4" t="inlineStr">
         <is>
           <t>71710175</t>
         </is>
       </c>
-      <c r="B122" s="11" t="inlineStr">
+      <c r="B122" s="5" t="inlineStr">
         <is>
           <t>INFANTES FERNANDEZ</t>
         </is>
       </c>
-      <c r="C122" s="11" t="inlineStr">
+      <c r="C122" s="5" t="inlineStr">
         <is>
           <t>BRANDOM VALDEMAR</t>
         </is>
       </c>
-      <c r="D122" s="11" t="inlineStr">
+      <c r="D122" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E122" s="11" t="inlineStr">
+      <c r="E122" s="5" t="inlineStr">
         <is>
           <t>Maquinaria Pesada</t>
         </is>
       </c>
-      <c r="F122" s="12" t="inlineStr">
+      <c r="F122" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G122" s="12" t="inlineStr">
+      <c r="G122" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H122" s="12" t="inlineStr">
+      <c r="H122" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I122" s="12" t="inlineStr">
+      <c r="I122" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J122" s="12" t="inlineStr">
+      <c r="J122" s="6" t="inlineStr">
         <is>
           <t>16:54</t>
         </is>
       </c>
-      <c r="K122" s="12" t="inlineStr">
+      <c r="K122" s="6" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="L122" s="12" t="inlineStr">
+      <c r="L122" s="6" t="inlineStr">
         <is>
           <t>01:00</t>
         </is>
       </c>
-      <c r="M122" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N122" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O122" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P122" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q122" s="12" t="inlineStr">
+      <c r="M122" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N122" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O122" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P122" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q122" s="6" t="inlineStr">
         <is>
           <t>08:01</t>
         </is>
       </c>
-      <c r="R122" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S122" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T122" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U122" s="12" t="inlineStr">
+      <c r="R122" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S122" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T122" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U122" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V122" s="11" t="inlineStr"/>
+      <c r="V122" s="5" t="inlineStr"/>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="4" t="inlineStr">
@@ -13846,112 +13846,112 @@
       <c r="V125" s="5" t="inlineStr"/>
     </row>
     <row r="126" ht="20" customHeight="1">
-      <c r="A126" s="10" t="inlineStr">
+      <c r="A126" s="4" t="inlineStr">
         <is>
           <t>72441086</t>
         </is>
       </c>
-      <c r="B126" s="11" t="inlineStr">
+      <c r="B126" s="5" t="inlineStr">
         <is>
           <t>BERMEO CRUZ</t>
         </is>
       </c>
-      <c r="C126" s="11" t="inlineStr">
+      <c r="C126" s="5" t="inlineStr">
         <is>
           <t>LLAMYR YASER</t>
         </is>
       </c>
-      <c r="D126" s="11" t="inlineStr">
+      <c r="D126" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E126" s="11" t="inlineStr">
+      <c r="E126" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F126" s="12" t="inlineStr">
+      <c r="F126" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G126" s="12" t="inlineStr">
+      <c r="G126" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H126" s="12" t="inlineStr">
+      <c r="H126" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I126" s="12" t="inlineStr">
+      <c r="I126" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J126" s="12" t="inlineStr">
+      <c r="J126" s="6" t="inlineStr">
         <is>
           <t>18:40</t>
         </is>
       </c>
-      <c r="K126" s="12" t="inlineStr">
+      <c r="K126" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L126" s="12" t="inlineStr">
+      <c r="L126" s="6" t="inlineStr">
         <is>
           <t>05:01</t>
         </is>
       </c>
-      <c r="M126" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N126" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O126" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P126" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q126" s="12" t="inlineStr">
+      <c r="M126" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N126" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O126" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P126" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q126" s="6" t="inlineStr">
         <is>
           <t>10:02</t>
         </is>
       </c>
-      <c r="R126" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S126" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T126" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U126" s="12" t="inlineStr">
+      <c r="R126" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S126" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T126" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U126" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V126" s="11" t="inlineStr"/>
+      <c r="V126" s="5" t="inlineStr"/>
     </row>
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="4" t="inlineStr">
@@ -14502,112 +14502,112 @@
       <c r="V131" s="5" t="inlineStr"/>
     </row>
     <row r="132" ht="20" customHeight="1">
-      <c r="A132" s="10" t="inlineStr">
+      <c r="A132" s="4" t="inlineStr">
         <is>
           <t>72500789</t>
         </is>
       </c>
-      <c r="B132" s="11" t="inlineStr">
+      <c r="B132" s="5" t="inlineStr">
         <is>
           <t>SAMBRANO QUISPESIVANA</t>
         </is>
       </c>
-      <c r="C132" s="11" t="inlineStr">
+      <c r="C132" s="5" t="inlineStr">
         <is>
           <t>ROY IVAN</t>
         </is>
       </c>
-      <c r="D132" s="11" t="inlineStr">
+      <c r="D132" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E132" s="11" t="inlineStr">
+      <c r="E132" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F132" s="12" t="inlineStr">
+      <c r="F132" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G132" s="12" t="inlineStr">
+      <c r="G132" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H132" s="12" t="inlineStr">
+      <c r="H132" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I132" s="12" t="inlineStr">
+      <c r="I132" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J132" s="12" t="inlineStr">
+      <c r="J132" s="6" t="inlineStr">
         <is>
           <t>04:56</t>
         </is>
       </c>
-      <c r="K132" s="12" t="inlineStr">
+      <c r="K132" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L132" s="12" t="inlineStr">
+      <c r="L132" s="6" t="inlineStr">
         <is>
           <t>16:51</t>
         </is>
       </c>
-      <c r="M132" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N132" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O132" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P132" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q132" s="12" t="inlineStr">
+      <c r="M132" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N132" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O132" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P132" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q132" s="6" t="inlineStr">
         <is>
           <t>11:51</t>
         </is>
       </c>
-      <c r="R132" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S132" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T132" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U132" s="12" t="inlineStr">
+      <c r="R132" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S132" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T132" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U132" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V132" s="11" t="inlineStr"/>
+      <c r="V132" s="5" t="inlineStr"/>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="4" t="inlineStr">
@@ -14718,112 +14718,112 @@
       <c r="V133" s="5" t="inlineStr"/>
     </row>
     <row r="134" ht="20" customHeight="1">
-      <c r="A134" s="10" t="inlineStr">
+      <c r="A134" s="4" t="inlineStr">
         <is>
           <t>72909375</t>
         </is>
       </c>
-      <c r="B134" s="11" t="inlineStr">
+      <c r="B134" s="5" t="inlineStr">
         <is>
           <t>BERMEO OJEDA</t>
         </is>
       </c>
-      <c r="C134" s="11" t="inlineStr">
+      <c r="C134" s="5" t="inlineStr">
         <is>
           <t>MANUEL GREGORIO</t>
         </is>
       </c>
-      <c r="D134" s="11" t="inlineStr">
+      <c r="D134" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E134" s="11" t="inlineStr">
+      <c r="E134" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F134" s="12" t="inlineStr">
+      <c r="F134" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G134" s="12" t="inlineStr">
+      <c r="G134" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H134" s="12" t="inlineStr">
+      <c r="H134" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I134" s="12" t="inlineStr">
+      <c r="I134" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J134" s="12" t="inlineStr">
+      <c r="J134" s="6" t="inlineStr">
         <is>
           <t>18:35</t>
         </is>
       </c>
-      <c r="K134" s="12" t="inlineStr">
+      <c r="K134" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L134" s="12" t="inlineStr">
+      <c r="L134" s="6" t="inlineStr">
         <is>
           <t>05:05</t>
         </is>
       </c>
-      <c r="M134" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N134" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O134" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P134" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q134" s="12" t="inlineStr">
+      <c r="M134" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N134" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O134" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P134" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q134" s="6" t="inlineStr">
         <is>
           <t>10:05</t>
         </is>
       </c>
-      <c r="R134" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S134" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T134" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U134" s="12" t="inlineStr">
+      <c r="R134" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S134" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T134" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U134" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V134" s="11" t="inlineStr"/>
+      <c r="V134" s="5" t="inlineStr"/>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="10" t="inlineStr">
@@ -15374,112 +15374,112 @@
       <c r="V139" s="5" t="inlineStr"/>
     </row>
     <row r="140" ht="20" customHeight="1">
-      <c r="A140" s="10" t="inlineStr">
+      <c r="A140" s="4" t="inlineStr">
         <is>
           <t>72940900</t>
         </is>
       </c>
-      <c r="B140" s="11" t="inlineStr">
+      <c r="B140" s="5" t="inlineStr">
         <is>
           <t>NOLE LADINES</t>
         </is>
       </c>
-      <c r="C140" s="11" t="inlineStr">
+      <c r="C140" s="5" t="inlineStr">
         <is>
           <t>CARLOS SEBASTIAN</t>
         </is>
       </c>
-      <c r="D140" s="11" t="inlineStr">
+      <c r="D140" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E140" s="11" t="inlineStr">
+      <c r="E140" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F140" s="12" t="inlineStr">
+      <c r="F140" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G140" s="12" t="inlineStr">
+      <c r="G140" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H140" s="12" t="inlineStr">
+      <c r="H140" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I140" s="12" t="inlineStr">
+      <c r="I140" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J140" s="12" t="inlineStr">
+      <c r="J140" s="6" t="inlineStr">
         <is>
           <t>04:51</t>
         </is>
       </c>
-      <c r="K140" s="12" t="inlineStr">
+      <c r="K140" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L140" s="12" t="inlineStr">
+      <c r="L140" s="6" t="inlineStr">
         <is>
           <t>16:50</t>
         </is>
       </c>
-      <c r="M140" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N140" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O140" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P140" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q140" s="12" t="inlineStr">
+      <c r="M140" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N140" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O140" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P140" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q140" s="6" t="inlineStr">
         <is>
           <t>11:51</t>
         </is>
       </c>
-      <c r="R140" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S140" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T140" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U140" s="12" t="inlineStr">
+      <c r="R140" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S140" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T140" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U140" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V140" s="11" t="inlineStr"/>
+      <c r="V140" s="5" t="inlineStr"/>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="4" t="inlineStr">
@@ -15698,112 +15698,112 @@
       <c r="V142" s="5" t="inlineStr"/>
     </row>
     <row r="143" ht="20" customHeight="1">
-      <c r="A143" s="10" t="inlineStr">
+      <c r="A143" s="4" t="inlineStr">
         <is>
           <t>72940901</t>
         </is>
       </c>
-      <c r="B143" s="11" t="inlineStr">
+      <c r="B143" s="5" t="inlineStr">
         <is>
           <t>NOLE LADINES</t>
         </is>
       </c>
-      <c r="C143" s="11" t="inlineStr">
+      <c r="C143" s="5" t="inlineStr">
         <is>
           <t>DIEGO ARMANDO</t>
         </is>
       </c>
-      <c r="D143" s="11" t="inlineStr">
+      <c r="D143" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E143" s="11" t="inlineStr">
+      <c r="E143" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F143" s="12" t="inlineStr">
+      <c r="F143" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G143" s="12" t="inlineStr">
+      <c r="G143" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H143" s="12" t="inlineStr">
+      <c r="H143" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I143" s="12" t="inlineStr">
+      <c r="I143" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J143" s="12" t="inlineStr">
+      <c r="J143" s="6" t="inlineStr">
         <is>
           <t>04:58</t>
         </is>
       </c>
-      <c r="K143" s="12" t="inlineStr">
+      <c r="K143" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L143" s="12" t="inlineStr">
+      <c r="L143" s="6" t="inlineStr">
         <is>
           <t>16:50</t>
         </is>
       </c>
-      <c r="M143" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N143" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O143" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P143" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q143" s="12" t="inlineStr">
+      <c r="M143" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N143" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O143" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P143" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q143" s="6" t="inlineStr">
         <is>
           <t>11:51</t>
         </is>
       </c>
-      <c r="R143" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S143" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T143" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U143" s="12" t="inlineStr">
+      <c r="R143" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S143" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T143" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U143" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V143" s="11" t="inlineStr"/>
+      <c r="V143" s="5" t="inlineStr"/>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="7" t="inlineStr">
@@ -16462,112 +16462,112 @@
       <c r="V149" s="5" t="inlineStr"/>
     </row>
     <row r="150" ht="20" customHeight="1">
-      <c r="A150" s="10" t="inlineStr">
+      <c r="A150" s="4" t="inlineStr">
         <is>
           <t>74070928</t>
         </is>
       </c>
-      <c r="B150" s="11" t="inlineStr">
+      <c r="B150" s="5" t="inlineStr">
         <is>
           <t>LEYVA ALAYO</t>
         </is>
       </c>
-      <c r="C150" s="11" t="inlineStr">
+      <c r="C150" s="5" t="inlineStr">
         <is>
           <t>LUIS DAVID</t>
         </is>
       </c>
-      <c r="D150" s="11" t="inlineStr">
+      <c r="D150" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E150" s="11" t="inlineStr">
+      <c r="E150" s="5" t="inlineStr">
         <is>
           <t>Maquinaria Pesada</t>
         </is>
       </c>
-      <c r="F150" s="12" t="inlineStr">
+      <c r="F150" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G150" s="12" t="inlineStr">
+      <c r="G150" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H150" s="12" t="inlineStr">
+      <c r="H150" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I150" s="12" t="inlineStr">
+      <c r="I150" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J150" s="12" t="inlineStr">
+      <c r="J150" s="6" t="inlineStr">
         <is>
           <t>05:02</t>
         </is>
       </c>
-      <c r="K150" s="12" t="inlineStr">
+      <c r="K150" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L150" s="12" t="inlineStr">
+      <c r="L150" s="6" t="inlineStr">
         <is>
           <t>16:53</t>
         </is>
       </c>
-      <c r="M150" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N150" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O150" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P150" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q150" s="12" t="inlineStr">
+      <c r="M150" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N150" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O150" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P150" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q150" s="6" t="inlineStr">
         <is>
           <t>11:52</t>
         </is>
       </c>
-      <c r="R150" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S150" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T150" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U150" s="12" t="inlineStr">
+      <c r="R150" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S150" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T150" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U150" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V150" s="11" t="inlineStr"/>
+      <c r="V150" s="5" t="inlineStr"/>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="4" t="inlineStr">
@@ -17438,112 +17438,112 @@
       <c r="V158" s="5" t="inlineStr"/>
     </row>
     <row r="159" ht="20" customHeight="1">
-      <c r="A159" s="10" t="inlineStr">
+      <c r="A159" s="4" t="inlineStr">
         <is>
           <t>75464754</t>
         </is>
       </c>
-      <c r="B159" s="11" t="inlineStr">
+      <c r="B159" s="5" t="inlineStr">
         <is>
           <t>CASANA VÁSQUEZ</t>
         </is>
       </c>
-      <c r="C159" s="11" t="inlineStr">
+      <c r="C159" s="5" t="inlineStr">
         <is>
           <t>JOSÉ GERONIMO</t>
         </is>
       </c>
-      <c r="D159" s="11" t="inlineStr">
+      <c r="D159" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E159" s="11" t="inlineStr">
+      <c r="E159" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F159" s="12" t="inlineStr">
+      <c r="F159" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G159" s="12" t="inlineStr">
+      <c r="G159" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H159" s="12" t="inlineStr">
+      <c r="H159" s="6" t="inlineStr">
         <is>
           <t>DIA</t>
         </is>
       </c>
-      <c r="I159" s="12" t="inlineStr">
+      <c r="I159" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J159" s="12" t="inlineStr">
+      <c r="J159" s="6" t="inlineStr">
         <is>
           <t>04:57</t>
         </is>
       </c>
-      <c r="K159" s="12" t="inlineStr">
+      <c r="K159" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L159" s="12" t="inlineStr">
+      <c r="L159" s="6" t="inlineStr">
         <is>
           <t>16:52</t>
         </is>
       </c>
-      <c r="M159" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N159" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O159" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P159" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q159" s="12" t="inlineStr">
+      <c r="M159" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N159" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O159" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P159" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q159" s="6" t="inlineStr">
         <is>
           <t>11:52</t>
         </is>
       </c>
-      <c r="R159" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S159" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T159" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U159" s="12" t="inlineStr">
+      <c r="R159" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S159" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T159" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U159" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V159" s="11" t="inlineStr"/>
+      <c r="V159" s="5" t="inlineStr"/>
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="10" t="inlineStr">
@@ -19502,220 +19502,220 @@
       <c r="V177" s="5" t="inlineStr"/>
     </row>
     <row r="178" ht="20" customHeight="1">
-      <c r="A178" s="10" t="inlineStr">
+      <c r="A178" s="4" t="inlineStr">
         <is>
           <t>77386038</t>
         </is>
       </c>
-      <c r="B178" s="11" t="inlineStr">
+      <c r="B178" s="5" t="inlineStr">
         <is>
           <t>RIMARACHIN GARCIA</t>
         </is>
       </c>
-      <c r="C178" s="11" t="inlineStr">
+      <c r="C178" s="5" t="inlineStr">
         <is>
           <t>CESAR</t>
         </is>
       </c>
-      <c r="D178" s="11" t="inlineStr">
+      <c r="D178" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E178" s="11" t="inlineStr">
+      <c r="E178" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F178" s="12" t="inlineStr">
+      <c r="F178" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G178" s="12" t="inlineStr">
+      <c r="G178" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H178" s="12" t="inlineStr">
+      <c r="H178" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I178" s="12" t="inlineStr">
+      <c r="I178" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J178" s="12" t="inlineStr">
+      <c r="J178" s="6" t="inlineStr">
         <is>
           <t>18:31</t>
         </is>
       </c>
-      <c r="K178" s="12" t="inlineStr">
+      <c r="K178" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L178" s="12" t="inlineStr">
+      <c r="L178" s="6" t="inlineStr">
         <is>
           <t>05:01</t>
         </is>
       </c>
-      <c r="M178" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N178" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O178" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P178" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q178" s="12" t="inlineStr">
+      <c r="M178" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N178" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O178" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P178" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q178" s="6" t="inlineStr">
         <is>
           <t>10:02</t>
         </is>
       </c>
-      <c r="R178" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S178" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T178" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U178" s="12" t="inlineStr">
+      <c r="R178" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S178" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T178" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U178" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V178" s="11" t="inlineStr"/>
+      <c r="V178" s="5" t="inlineStr"/>
     </row>
     <row r="179" ht="20" customHeight="1">
-      <c r="A179" s="10" t="inlineStr">
+      <c r="A179" s="4" t="inlineStr">
         <is>
           <t>77386038</t>
         </is>
       </c>
-      <c r="B179" s="11" t="inlineStr">
+      <c r="B179" s="5" t="inlineStr">
         <is>
           <t>RIMARACHIN GARCIA</t>
         </is>
       </c>
-      <c r="C179" s="11" t="inlineStr">
+      <c r="C179" s="5" t="inlineStr">
         <is>
           <t>CESAR</t>
         </is>
       </c>
-      <c r="D179" s="11" t="inlineStr">
+      <c r="D179" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E179" s="11" t="inlineStr">
+      <c r="E179" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F179" s="12" t="inlineStr">
+      <c r="F179" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G179" s="12" t="inlineStr">
+      <c r="G179" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H179" s="12" t="inlineStr">
+      <c r="H179" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I179" s="12" t="inlineStr">
+      <c r="I179" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J179" s="12" t="inlineStr">
+      <c r="J179" s="6" t="inlineStr">
         <is>
           <t>16:50</t>
         </is>
       </c>
-      <c r="K179" s="12" t="inlineStr">
+      <c r="K179" s="6" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="L179" s="12" t="inlineStr">
+      <c r="L179" s="6" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="M179" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N179" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O179" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P179" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q179" s="12" t="inlineStr">
+      <c r="M179" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N179" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O179" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P179" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q179" s="6" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="R179" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S179" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T179" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U179" s="12" t="inlineStr">
+      <c r="R179" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S179" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T179" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U179" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V179" s="11" t="inlineStr"/>
+      <c r="V179" s="5" t="inlineStr"/>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="10" t="inlineStr">
@@ -20046,220 +20046,220 @@
       <c r="V182" s="5" t="inlineStr"/>
     </row>
     <row r="183" ht="20" customHeight="1">
-      <c r="A183" s="10" t="inlineStr">
+      <c r="A183" s="4" t="inlineStr">
         <is>
           <t>78197802</t>
         </is>
       </c>
-      <c r="B183" s="11" t="inlineStr">
+      <c r="B183" s="5" t="inlineStr">
         <is>
           <t>NEYRA CAMPOS</t>
         </is>
       </c>
-      <c r="C183" s="11" t="inlineStr">
+      <c r="C183" s="5" t="inlineStr">
         <is>
           <t>YULEISER</t>
         </is>
       </c>
-      <c r="D183" s="11" t="inlineStr">
+      <c r="D183" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E183" s="11" t="inlineStr">
+      <c r="E183" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F183" s="12" t="inlineStr">
+      <c r="F183" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="G183" s="12" t="inlineStr">
+      <c r="G183" s="6" t="inlineStr">
         <is>
           <t>Martes</t>
         </is>
       </c>
-      <c r="H183" s="12" t="inlineStr">
+      <c r="H183" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I183" s="12" t="inlineStr">
+      <c r="I183" s="6" t="inlineStr">
         <is>
           <t>18/08/2026</t>
         </is>
       </c>
-      <c r="J183" s="12" t="inlineStr">
+      <c r="J183" s="6" t="inlineStr">
         <is>
           <t>18:31</t>
         </is>
       </c>
-      <c r="K183" s="12" t="inlineStr">
+      <c r="K183" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="L183" s="12" t="inlineStr">
+      <c r="L183" s="6" t="inlineStr">
         <is>
           <t>05:01</t>
         </is>
       </c>
-      <c r="M183" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N183" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O183" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P183" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q183" s="12" t="inlineStr">
+      <c r="M183" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N183" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O183" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P183" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q183" s="6" t="inlineStr">
         <is>
           <t>10:02</t>
         </is>
       </c>
-      <c r="R183" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S183" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T183" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U183" s="12" t="inlineStr">
+      <c r="R183" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S183" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T183" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U183" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V183" s="11" t="inlineStr"/>
+      <c r="V183" s="5" t="inlineStr"/>
     </row>
     <row r="184" ht="20" customHeight="1">
-      <c r="A184" s="10" t="inlineStr">
+      <c r="A184" s="4" t="inlineStr">
         <is>
           <t>78197802</t>
         </is>
       </c>
-      <c r="B184" s="11" t="inlineStr">
+      <c r="B184" s="5" t="inlineStr">
         <is>
           <t>NEYRA CAMPOS</t>
         </is>
       </c>
-      <c r="C184" s="11" t="inlineStr">
+      <c r="C184" s="5" t="inlineStr">
         <is>
           <t>YULEISER</t>
         </is>
       </c>
-      <c r="D184" s="11" t="inlineStr">
+      <c r="D184" s="5" t="inlineStr">
         <is>
           <t>Oper&amp;Mtto</t>
         </is>
       </c>
-      <c r="E184" s="11" t="inlineStr">
+      <c r="E184" s="5" t="inlineStr">
         <is>
           <t>Operaciones</t>
         </is>
       </c>
-      <c r="F184" s="12" t="inlineStr">
+      <c r="F184" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="G184" s="12" t="inlineStr">
+      <c r="G184" s="6" t="inlineStr">
         <is>
           <t>Miércoles</t>
         </is>
       </c>
-      <c r="H184" s="12" t="inlineStr">
+      <c r="H184" s="6" t="inlineStr">
         <is>
           <t>NOCHE</t>
         </is>
       </c>
-      <c r="I184" s="12" t="inlineStr">
+      <c r="I184" s="6" t="inlineStr">
         <is>
           <t>19/08/2026</t>
         </is>
       </c>
-      <c r="J184" s="12" t="inlineStr">
+      <c r="J184" s="6" t="inlineStr">
         <is>
           <t>16:32</t>
         </is>
       </c>
-      <c r="K184" s="12" t="inlineStr">
+      <c r="K184" s="6" t="inlineStr">
         <is>
           <t>20/08/2026</t>
         </is>
       </c>
-      <c r="L184" s="12" t="inlineStr">
+      <c r="L184" s="6" t="inlineStr">
         <is>
           <t>07:04</t>
         </is>
       </c>
-      <c r="M184" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N184" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O184" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P184" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q184" s="12" t="inlineStr">
+      <c r="M184" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N184" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O184" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P184" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q184" s="6" t="inlineStr">
         <is>
           <t>14:05</t>
         </is>
       </c>
-      <c r="R184" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="S184" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T184" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U184" s="12" t="inlineStr">
+      <c r="R184" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S184" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T184" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U184" s="6" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V184" s="11" t="inlineStr"/>
+      <c r="V184" s="5" t="inlineStr"/>
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="10" t="inlineStr">

</xml_diff>

<commit_message>
fix: Capitalized J in Exceso de Jornada, set Tipo Registro to Horas extras when both excess and HE exist, and formatted Jornada Parcial obs as Cambio de guardia (Medio dia) (hh:mm)
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -1637,7 +1637,7 @@
       </c>
       <c r="V13" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:01)</t>
+          <t>Cambio de guardia (Medio día) (06:01)</t>
         </is>
       </c>
     </row>
@@ -2068,12 +2068,12 @@
       </c>
       <c r="U17" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V17" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:56)</t>
+          <t>Exceso de Jornada (01:56)</t>
         </is>
       </c>
     </row>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="V29" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:02)</t>
+          <t>Cambio de guardia (Medio día) (06:02)</t>
         </is>
       </c>
     </row>
@@ -5884,12 +5884,12 @@
       </c>
       <c r="U52" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada/Horas Extras</t>
+          <t>Horas extras</t>
         </is>
       </c>
       <c r="V52" s="5" t="inlineStr">
         <is>
-          <t>Horas extras (01:40), Exceso de jornada (01:10), Tardanza (00:02)</t>
+          <t>Horas extras (01:40), Exceso de Jornada (01:10), Tardanza (00:02)</t>
         </is>
       </c>
     </row>
@@ -6752,12 +6752,12 @@
       </c>
       <c r="U60" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V60" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (02:42), Entrada duplicada (06:40)</t>
+          <t>Exceso de Jornada (02:42), Entrada duplicada (06:40)</t>
         </is>
       </c>
     </row>
@@ -6976,12 +6976,12 @@
       </c>
       <c r="U62" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V62" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (00:30)</t>
+          <t>Exceso de Jornada (00:30)</t>
         </is>
       </c>
     </row>
@@ -7192,12 +7192,12 @@
       </c>
       <c r="U64" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V64" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:11)</t>
+          <t>Exceso de Jornada (01:11)</t>
         </is>
       </c>
     </row>
@@ -7304,12 +7304,12 @@
       </c>
       <c r="U65" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V65" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:11)</t>
+          <t>Exceso de Jornada (01:11)</t>
         </is>
       </c>
     </row>
@@ -7416,12 +7416,12 @@
       </c>
       <c r="U66" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V66" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (03:26)</t>
+          <t>Exceso de Jornada (03:26)</t>
         </is>
       </c>
     </row>
@@ -7528,12 +7528,12 @@
       </c>
       <c r="U67" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V67" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (00:47)</t>
+          <t>Exceso de Jornada (00:47)</t>
         </is>
       </c>
     </row>
@@ -8617,7 +8617,7 @@
       </c>
       <c r="V77" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:12)</t>
+          <t>Cambio de guardia (Medio día) (06:12)</t>
         </is>
       </c>
     </row>
@@ -8832,12 +8832,12 @@
       </c>
       <c r="U79" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V79" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:18)</t>
+          <t>Exceso de Jornada (01:18)</t>
         </is>
       </c>
     </row>
@@ -8944,12 +8944,12 @@
       </c>
       <c r="U80" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V80" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (02:38)</t>
+          <t>Exceso de Jornada (02:38)</t>
         </is>
       </c>
     </row>
@@ -9817,7 +9817,7 @@
       </c>
       <c r="V88" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (05:43), Entrada duplicada (07:17, 07:18), Tardanza (00:02)</t>
+          <t>Cambio de guardia (Medio día) (05:43), Entrada duplicada (07:17, 07:18), Tardanza (00:02)</t>
         </is>
       </c>
     </row>
@@ -10032,12 +10032,12 @@
       </c>
       <c r="U90" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V90" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:17)</t>
+          <t>Exceso de Jornada (01:17)</t>
         </is>
       </c>
     </row>
@@ -10144,12 +10144,12 @@
       </c>
       <c r="U91" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V91" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (02:38)</t>
+          <t>Exceso de Jornada (02:38)</t>
         </is>
       </c>
     </row>
@@ -10913,7 +10913,7 @@
       </c>
       <c r="V98" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:15)</t>
+          <t>Cambio de guardia (Medio día) (06:15)</t>
         </is>
       </c>
     </row>
@@ -11673,7 +11673,7 @@
       </c>
       <c r="V105" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:07)</t>
+          <t>Cambio de guardia (Medio día) (06:07)</t>
         </is>
       </c>
     </row>
@@ -11785,7 +11785,7 @@
       </c>
       <c r="V106" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (05:55)</t>
+          <t>Cambio de guardia (Medio día) (05:55)</t>
         </is>
       </c>
     </row>
@@ -13085,7 +13085,7 @@
       </c>
       <c r="V118" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:12)</t>
+          <t>Cambio de guardia (Medio día) (06:12)</t>
         </is>
       </c>
     </row>
@@ -14056,12 +14056,12 @@
       </c>
       <c r="U127" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada/Tardanza</t>
+          <t>Exceso de Jornada/Tardanza</t>
         </is>
       </c>
       <c r="V127" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:13), Tardanza (00:33)</t>
+          <t>Exceso de Jornada (01:13), Tardanza (00:33)</t>
         </is>
       </c>
     </row>
@@ -14173,7 +14173,7 @@
       </c>
       <c r="V128" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:09)</t>
+          <t>Cambio de guardia (Medio día) (06:09)</t>
         </is>
       </c>
     </row>
@@ -14933,7 +14933,7 @@
       </c>
       <c r="V135" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (07:55)</t>
+          <t>Cambio de guardia (Medio día) (07:55)</t>
         </is>
       </c>
     </row>
@@ -15045,7 +15045,7 @@
       </c>
       <c r="V136" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:00)</t>
+          <t>Cambio de guardia (Medio día) (06:00)</t>
         </is>
       </c>
     </row>
@@ -16128,12 +16128,12 @@
       </c>
       <c r="U146" s="6" t="inlineStr">
         <is>
-          <t>Exceso de jornada</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="V146" s="5" t="inlineStr">
         <is>
-          <t>Exceso de jornada (01:23)</t>
+          <t>Exceso de Jornada (01:23)</t>
         </is>
       </c>
     </row>
@@ -17653,7 +17653,7 @@
       </c>
       <c r="V160" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (05:51)</t>
+          <t>Cambio de guardia (Medio día) (05:51)</t>
         </is>
       </c>
     </row>
@@ -19825,7 +19825,7 @@
       </c>
       <c r="V180" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:26)</t>
+          <t>Cambio de guardia (Medio día) (06:26)</t>
         </is>
       </c>
     </row>
@@ -20369,7 +20369,7 @@
       </c>
       <c r="V185" s="11" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:25)</t>
+          <t>Cambio de guardia (Medio día) (06:25)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Set Column U to Cambio de guardia and Column V to Jornada parcial (Medio dia) (hh:mm)
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -1632,12 +1632,12 @@
       </c>
       <c r="U13" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V13" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:01)</t>
+          <t>Jornada parcial (Medio día) (06:01)</t>
         </is>
       </c>
     </row>
@@ -3384,12 +3384,12 @@
       </c>
       <c r="U29" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V29" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:02)</t>
+          <t>Jornada parcial (Medio día) (06:02)</t>
         </is>
       </c>
     </row>
@@ -8612,12 +8612,12 @@
       </c>
       <c r="U77" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V77" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:12)</t>
+          <t>Jornada parcial (Medio día) (06:12)</t>
         </is>
       </c>
     </row>
@@ -9812,12 +9812,12 @@
       </c>
       <c r="U88" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V88" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (05:43), Entrada duplicada (07:17, 07:18), Tardanza (00:02)</t>
+          <t>Jornada parcial (Medio día) (05:43), Entrada duplicada (07:17, 07:18), Tardanza (00:02)</t>
         </is>
       </c>
     </row>
@@ -10908,12 +10908,12 @@
       </c>
       <c r="U98" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V98" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:15)</t>
+          <t>Jornada parcial (Medio día) (06:15)</t>
         </is>
       </c>
     </row>
@@ -11668,12 +11668,12 @@
       </c>
       <c r="U105" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V105" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:07)</t>
+          <t>Jornada parcial (Medio día) (06:07)</t>
         </is>
       </c>
     </row>
@@ -11780,12 +11780,12 @@
       </c>
       <c r="U106" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V106" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (05:55)</t>
+          <t>Jornada parcial (Medio día) (05:55)</t>
         </is>
       </c>
     </row>
@@ -13080,12 +13080,12 @@
       </c>
       <c r="U118" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V118" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:12)</t>
+          <t>Jornada parcial (Medio día) (06:12)</t>
         </is>
       </c>
     </row>
@@ -14168,12 +14168,12 @@
       </c>
       <c r="U128" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V128" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:09)</t>
+          <t>Jornada parcial (Medio día) (06:09)</t>
         </is>
       </c>
     </row>
@@ -14928,12 +14928,12 @@
       </c>
       <c r="U135" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V135" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (07:55)</t>
+          <t>Jornada parcial (Medio día) (07:55)</t>
         </is>
       </c>
     </row>
@@ -15040,12 +15040,12 @@
       </c>
       <c r="U136" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V136" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:00)</t>
+          <t>Jornada parcial (Medio día) (06:00)</t>
         </is>
       </c>
     </row>
@@ -17648,12 +17648,12 @@
       </c>
       <c r="U160" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V160" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (05:51)</t>
+          <t>Jornada parcial (Medio día) (05:51)</t>
         </is>
       </c>
     </row>
@@ -19820,12 +19820,12 @@
       </c>
       <c r="U180" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V180" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:26)</t>
+          <t>Jornada parcial (Medio día) (06:26)</t>
         </is>
       </c>
     </row>
@@ -20364,12 +20364,12 @@
       </c>
       <c r="U185" s="12" t="inlineStr">
         <is>
-          <t>Jornada parcial</t>
+          <t>Cambio de guardia</t>
         </is>
       </c>
       <c r="V185" s="11" t="inlineStr">
         <is>
-          <t>Cambio de guardia (Medio día) (06:25)</t>
+          <t>Jornada parcial (Medio día) (06:25)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Restructured Excel report to 23 columns (A to W), inserted Horas Extras column, and renamed headers
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -529,12 +529,13 @@
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
     <col width="15" customWidth="1" min="16" max="16"/>
-    <col width="25" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="22" customWidth="1" min="21" max="21"/>
-    <col width="48" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="25" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="50" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -620,7 +621,7 @@
       </c>
       <c r="N4" s="3" t="inlineStr">
         <is>
-          <t>Hora Inicio H.E.</t>
+          <t>Inicio H.E.</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
@@ -630,40 +631,44 @@
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Hora Fin H.E.</t>
+          <t>Fin H.E.</t>
         </is>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>Horas Trabajadas (hh:mm)</t>
+          <t>Horas de Turno</t>
         </is>
       </c>
       <c r="R4" s="3" t="inlineStr">
         <is>
-          <t>Tardanza (hh:mm)</t>
+          <t>Exceso de Turno</t>
         </is>
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>Exceso Jornada (hh:mm)</t>
+          <t>Horas Extras</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Horas Extras Totales (hh:mm)</t>
+          <t>Total de Horas Adicionales</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
+          <t>Tardanza</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
           <t>Tipo Registro</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="W4" s="3" t="inlineStr">
         <is>
           <t>Observación / Incidencias</t>
         </is>
       </c>
-      <c r="W4" s="3" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -768,10 +773,15 @@
       </c>
       <c r="U5" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V5" s="5" t="inlineStr"/>
+      <c r="W5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -876,10 +886,15 @@
       </c>
       <c r="U6" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V6" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V6" s="5" t="inlineStr"/>
+      <c r="W6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -984,10 +999,15 @@
       </c>
       <c r="U7" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V7" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V7" s="5" t="inlineStr"/>
+      <c r="W7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -1088,10 +1108,15 @@
       </c>
       <c r="U8" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V8" s="9" t="inlineStr">
+        <is>
           <t>Entrada pendiente</t>
         </is>
       </c>
-      <c r="V8" s="8" t="inlineStr">
+      <c r="W8" s="8" t="inlineStr">
         <is>
           <t>Salida sin registro de entrada previa (19:11)</t>
         </is>
@@ -1196,10 +1221,15 @@
       </c>
       <c r="U9" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V9" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V9" s="8" t="inlineStr">
+      <c r="W9" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -1308,10 +1338,15 @@
       </c>
       <c r="U10" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V10" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V10" s="5" t="inlineStr"/>
+      <c r="W10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
@@ -1416,10 +1451,15 @@
       </c>
       <c r="U11" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V11" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V11" s="5" t="inlineStr"/>
+      <c r="W11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
@@ -1520,10 +1560,15 @@
       </c>
       <c r="U12" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V12" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V12" s="8" t="inlineStr">
+      <c r="W12" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -1632,10 +1677,15 @@
       </c>
       <c r="U13" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V13" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V13" s="11" t="inlineStr">
+      <c r="W13" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:01)</t>
         </is>
@@ -1744,10 +1794,15 @@
       </c>
       <c r="U14" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V14" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V14" s="5" t="inlineStr"/>
+      <c r="W14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1852,10 +1907,15 @@
       </c>
       <c r="U15" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V15" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V15" s="5" t="inlineStr"/>
+      <c r="W15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1960,10 +2020,15 @@
       </c>
       <c r="U16" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V16" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V16" s="5" t="inlineStr"/>
+      <c r="W16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
@@ -2053,25 +2118,30 @@
       </c>
       <c r="R17" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:56</t>
         </is>
       </c>
       <c r="S17" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T17" s="6" t="inlineStr">
+        <is>
           <t>01:56</t>
         </is>
       </c>
-      <c r="T17" s="6" t="inlineStr">
-        <is>
-          <t>01:56</t>
-        </is>
-      </c>
       <c r="U17" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V17" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V17" s="5" t="inlineStr">
+      <c r="W17" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:56)</t>
         </is>
@@ -2180,10 +2250,15 @@
       </c>
       <c r="U18" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V18" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V18" s="5" t="inlineStr"/>
+      <c r="W18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
@@ -2288,10 +2363,15 @@
       </c>
       <c r="U19" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V19" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V19" s="5" t="inlineStr"/>
+      <c r="W19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
@@ -2396,10 +2476,15 @@
       </c>
       <c r="U20" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V20" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V20" s="5" t="inlineStr"/>
+      <c r="W20" s="5" t="inlineStr"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -2500,10 +2585,15 @@
       </c>
       <c r="U21" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V21" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V21" s="8" t="inlineStr">
+      <c r="W21" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -2612,10 +2702,15 @@
       </c>
       <c r="U22" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V22" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V22" s="5" t="inlineStr">
+      <c r="W22" s="5" t="inlineStr">
         <is>
           <t>Entrada duplicada (18:41)</t>
         </is>
@@ -2720,10 +2815,15 @@
       </c>
       <c r="U23" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V23" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V23" s="8" t="inlineStr">
+      <c r="W23" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -2832,10 +2932,15 @@
       </c>
       <c r="U24" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V24" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V24" s="5" t="inlineStr"/>
+      <c r="W24" s="5" t="inlineStr"/>
     </row>
     <row r="25" ht="20" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
@@ -2940,10 +3045,15 @@
       </c>
       <c r="U25" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V25" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V25" s="5" t="inlineStr"/>
+      <c r="W25" s="5" t="inlineStr"/>
     </row>
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="7" t="inlineStr">
@@ -3048,10 +3158,15 @@
       </c>
       <c r="U26" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V26" s="9" t="inlineStr">
+        <is>
           <t>Salida anticipada</t>
         </is>
       </c>
-      <c r="V26" s="8" t="inlineStr">
+      <c r="W26" s="8" t="inlineStr">
         <is>
           <t>Salida anticipada (00:04)</t>
         </is>
@@ -3145,25 +3260,30 @@
       </c>
       <c r="R27" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S27" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T27" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U27" s="6" t="inlineStr">
+        <is>
           <t>00:57</t>
         </is>
       </c>
-      <c r="S27" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T27" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U27" s="6" t="inlineStr">
+      <c r="V27" s="6" t="inlineStr">
         <is>
           <t>Tardanza</t>
         </is>
       </c>
-      <c r="V27" s="5" t="inlineStr">
+      <c r="W27" s="5" t="inlineStr">
         <is>
           <t>Tardanza (00:57)</t>
         </is>
@@ -3272,10 +3392,15 @@
       </c>
       <c r="U28" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V28" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V28" s="5" t="inlineStr">
+      <c r="W28" s="5" t="inlineStr">
         <is>
           <t>Entrada duplicada (18:17)</t>
         </is>
@@ -3384,10 +3509,15 @@
       </c>
       <c r="U29" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V29" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V29" s="11" t="inlineStr">
+      <c r="W29" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:02)</t>
         </is>
@@ -3496,10 +3626,15 @@
       </c>
       <c r="U30" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V30" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V30" s="5" t="inlineStr"/>
+      <c r="W30" s="5" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
@@ -3604,10 +3739,15 @@
       </c>
       <c r="U31" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V31" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V31" s="5" t="inlineStr"/>
+      <c r="W31" s="5" t="inlineStr"/>
     </row>
     <row r="32" ht="20" customHeight="1">
       <c r="A32" s="4" t="inlineStr">
@@ -3712,10 +3852,15 @@
       </c>
       <c r="U32" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V32" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V32" s="5" t="inlineStr"/>
+      <c r="W32" s="5" t="inlineStr"/>
     </row>
     <row r="33" ht="20" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -3820,10 +3965,15 @@
       </c>
       <c r="U33" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V33" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V33" s="5" t="inlineStr"/>
+      <c r="W33" s="5" t="inlineStr"/>
     </row>
     <row r="34" ht="20" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
@@ -3928,10 +4078,15 @@
       </c>
       <c r="U34" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V34" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V34" s="5" t="inlineStr"/>
+      <c r="W34" s="5" t="inlineStr"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
@@ -4036,10 +4191,15 @@
       </c>
       <c r="U35" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V35" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V35" s="5" t="inlineStr"/>
+      <c r="W35" s="5" t="inlineStr"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="4" t="inlineStr">
@@ -4144,10 +4304,15 @@
       </c>
       <c r="U36" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V36" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V36" s="5" t="inlineStr"/>
+      <c r="W36" s="5" t="inlineStr"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="7" t="inlineStr">
@@ -4248,10 +4413,15 @@
       </c>
       <c r="U37" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V37" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V37" s="8" t="inlineStr">
+      <c r="W37" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -4356,10 +4526,15 @@
       </c>
       <c r="U38" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V38" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V38" s="8" t="inlineStr">
+      <c r="W38" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -4458,7 +4633,7 @@
       </c>
       <c r="S39" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="T39" s="6" t="inlineStr">
@@ -4468,10 +4643,15 @@
       </c>
       <c r="U39" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V39" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V39" s="5" t="inlineStr">
+      <c r="W39" s="5" t="inlineStr">
         <is>
           <t>Horas extras (04:00)</t>
         </is>
@@ -4570,7 +4750,7 @@
       </c>
       <c r="S40" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>03:53</t>
         </is>
       </c>
       <c r="T40" s="6" t="inlineStr">
@@ -4580,10 +4760,15 @@
       </c>
       <c r="U40" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V40" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V40" s="5" t="inlineStr">
+      <c r="W40" s="5" t="inlineStr">
         <is>
           <t>Horas extras (03:53)</t>
         </is>
@@ -4682,7 +4867,7 @@
       </c>
       <c r="S41" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>03:20</t>
         </is>
       </c>
       <c r="T41" s="6" t="inlineStr">
@@ -4692,10 +4877,15 @@
       </c>
       <c r="U41" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V41" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V41" s="5" t="inlineStr">
+      <c r="W41" s="5" t="inlineStr">
         <is>
           <t>Horas extras (03:20)</t>
         </is>
@@ -4794,7 +4984,7 @@
       </c>
       <c r="S42" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>04:50</t>
         </is>
       </c>
       <c r="T42" s="6" t="inlineStr">
@@ -4804,10 +4994,15 @@
       </c>
       <c r="U42" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V42" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V42" s="5" t="inlineStr">
+      <c r="W42" s="5" t="inlineStr">
         <is>
           <t>Horas extras (04:50)</t>
         </is>
@@ -4912,10 +5107,15 @@
       </c>
       <c r="U43" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V43" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V43" s="8" t="inlineStr">
+      <c r="W43" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -5024,10 +5224,15 @@
       </c>
       <c r="U44" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V44" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V44" s="5" t="inlineStr"/>
+      <c r="W44" s="5" t="inlineStr"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -5132,10 +5337,15 @@
       </c>
       <c r="U45" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V45" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V45" s="5" t="inlineStr"/>
+      <c r="W45" s="5" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="4" t="inlineStr">
@@ -5240,10 +5450,15 @@
       </c>
       <c r="U46" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V46" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V46" s="5" t="inlineStr"/>
+      <c r="W46" s="5" t="inlineStr"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
@@ -5348,10 +5563,15 @@
       </c>
       <c r="U47" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V47" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V47" s="5" t="inlineStr"/>
+      <c r="W47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="20" customHeight="1">
       <c r="A48" s="4" t="inlineStr">
@@ -5452,10 +5672,15 @@
       </c>
       <c r="U48" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V48" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V48" s="5" t="inlineStr"/>
+      <c r="W48" s="5" t="inlineStr"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -5560,10 +5785,15 @@
       </c>
       <c r="U49" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V49" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V49" s="5" t="inlineStr"/>
+      <c r="W49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="20" customHeight="1">
       <c r="A50" s="7" t="inlineStr">
@@ -5664,10 +5894,15 @@
       </c>
       <c r="U50" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V50" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V50" s="8" t="inlineStr">
+      <c r="W50" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -5776,10 +6011,15 @@
       </c>
       <c r="U51" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V51" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V51" s="5" t="inlineStr"/>
+      <c r="W51" s="5" t="inlineStr"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="4" t="inlineStr">
@@ -5869,25 +6109,30 @@
       </c>
       <c r="R52" s="6" t="inlineStr">
         <is>
+          <t>01:10</t>
+        </is>
+      </c>
+      <c r="S52" s="6" t="inlineStr">
+        <is>
+          <t>01:40</t>
+        </is>
+      </c>
+      <c r="T52" s="6" t="inlineStr">
+        <is>
+          <t>02:50</t>
+        </is>
+      </c>
+      <c r="U52" s="6" t="inlineStr">
+        <is>
           <t>00:02</t>
         </is>
       </c>
-      <c r="S52" s="6" t="inlineStr">
-        <is>
-          <t>01:10</t>
-        </is>
-      </c>
-      <c r="T52" s="6" t="inlineStr">
-        <is>
-          <t>02:50</t>
-        </is>
-      </c>
-      <c r="U52" s="6" t="inlineStr">
+      <c r="V52" s="6" t="inlineStr">
         <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V52" s="5" t="inlineStr">
+      <c r="W52" s="5" t="inlineStr">
         <is>
           <t>Horas extras (01:40), Exceso de Jornada (01:10), Tardanza (00:02)</t>
         </is>
@@ -5996,10 +6241,15 @@
       </c>
       <c r="U53" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V53" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V53" s="5" t="inlineStr"/>
+      <c r="W53" s="5" t="inlineStr"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="4" t="inlineStr">
@@ -6104,10 +6354,15 @@
       </c>
       <c r="U54" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V54" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V54" s="5" t="inlineStr"/>
+      <c r="W54" s="5" t="inlineStr"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
@@ -6208,10 +6463,15 @@
       </c>
       <c r="U55" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V55" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V55" s="8" t="inlineStr">
+      <c r="W55" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -6320,10 +6580,15 @@
       </c>
       <c r="U56" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V56" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V56" s="5" t="inlineStr"/>
+      <c r="W56" s="5" t="inlineStr"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -6428,10 +6693,15 @@
       </c>
       <c r="U57" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V57" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V57" s="5" t="inlineStr"/>
+      <c r="W57" s="5" t="inlineStr"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="4" t="inlineStr">
@@ -6536,10 +6806,15 @@
       </c>
       <c r="U58" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V58" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V58" s="5" t="inlineStr"/>
+      <c r="W58" s="5" t="inlineStr"/>
     </row>
     <row r="59" ht="20" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -6644,10 +6919,15 @@
       </c>
       <c r="U59" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V59" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V59" s="5" t="inlineStr"/>
+      <c r="W59" s="5" t="inlineStr"/>
     </row>
     <row r="60" ht="20" customHeight="1">
       <c r="A60" s="4" t="inlineStr">
@@ -6737,25 +7017,30 @@
       </c>
       <c r="R60" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:42</t>
         </is>
       </c>
       <c r="S60" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T60" s="6" t="inlineStr">
+        <is>
           <t>02:42</t>
         </is>
       </c>
-      <c r="T60" s="6" t="inlineStr">
-        <is>
-          <t>02:42</t>
-        </is>
-      </c>
       <c r="U60" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V60" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V60" s="5" t="inlineStr">
+      <c r="W60" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (02:42), Entrada duplicada (06:40)</t>
         </is>
@@ -6854,7 +7139,7 @@
       </c>
       <c r="S61" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:32</t>
         </is>
       </c>
       <c r="T61" s="6" t="inlineStr">
@@ -6864,10 +7149,15 @@
       </c>
       <c r="U61" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V61" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V61" s="5" t="inlineStr">
+      <c r="W61" s="5" t="inlineStr">
         <is>
           <t>Horas extras (02:32)</t>
         </is>
@@ -6961,25 +7251,30 @@
       </c>
       <c r="R62" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="S62" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T62" s="6" t="inlineStr">
+        <is>
           <t>00:30</t>
         </is>
       </c>
-      <c r="T62" s="6" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
       <c r="U62" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V62" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V62" s="5" t="inlineStr">
+      <c r="W62" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (00:30)</t>
         </is>
@@ -7084,10 +7379,15 @@
       </c>
       <c r="U63" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V63" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V63" s="8" t="inlineStr"/>
+      <c r="W63" s="8" t="inlineStr"/>
     </row>
     <row r="64" ht="20" customHeight="1">
       <c r="A64" s="4" t="inlineStr">
@@ -7177,25 +7477,30 @@
       </c>
       <c r="R64" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:11</t>
         </is>
       </c>
       <c r="S64" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T64" s="6" t="inlineStr">
+        <is>
           <t>01:11</t>
         </is>
       </c>
-      <c r="T64" s="6" t="inlineStr">
-        <is>
-          <t>01:11</t>
-        </is>
-      </c>
       <c r="U64" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V64" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V64" s="5" t="inlineStr">
+      <c r="W64" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:11)</t>
         </is>
@@ -7289,25 +7594,30 @@
       </c>
       <c r="R65" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:11</t>
         </is>
       </c>
       <c r="S65" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T65" s="6" t="inlineStr">
+        <is>
           <t>01:11</t>
         </is>
       </c>
-      <c r="T65" s="6" t="inlineStr">
-        <is>
-          <t>01:11</t>
-        </is>
-      </c>
       <c r="U65" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V65" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V65" s="5" t="inlineStr">
+      <c r="W65" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:11)</t>
         </is>
@@ -7401,25 +7711,30 @@
       </c>
       <c r="R66" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>03:26</t>
         </is>
       </c>
       <c r="S66" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T66" s="6" t="inlineStr">
+        <is>
           <t>03:26</t>
         </is>
       </c>
-      <c r="T66" s="6" t="inlineStr">
-        <is>
-          <t>03:26</t>
-        </is>
-      </c>
       <c r="U66" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V66" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V66" s="5" t="inlineStr">
+      <c r="W66" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (03:26)</t>
         </is>
@@ -7513,25 +7828,30 @@
       </c>
       <c r="R67" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:47</t>
         </is>
       </c>
       <c r="S67" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T67" s="6" t="inlineStr">
+        <is>
           <t>00:47</t>
         </is>
       </c>
-      <c r="T67" s="6" t="inlineStr">
-        <is>
-          <t>00:47</t>
-        </is>
-      </c>
       <c r="U67" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V67" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V67" s="5" t="inlineStr">
+      <c r="W67" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (00:47)</t>
         </is>
@@ -7636,10 +7956,15 @@
       </c>
       <c r="U68" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V68" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V68" s="8" t="inlineStr">
+      <c r="W68" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -7729,25 +8054,30 @@
       </c>
       <c r="R69" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S69" s="9" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T69" s="9" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U69" s="9" t="inlineStr">
+        <is>
           <t>00:05</t>
         </is>
       </c>
-      <c r="S69" s="9" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T69" s="9" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U69" s="9" t="inlineStr">
+      <c r="V69" s="9" t="inlineStr">
         <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V69" s="8" t="inlineStr">
+      <c r="W69" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida, Tardanza (00:05)</t>
         </is>
@@ -7856,10 +8186,15 @@
       </c>
       <c r="U70" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V70" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V70" s="5" t="inlineStr"/>
+      <c r="W70" s="5" t="inlineStr"/>
     </row>
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
@@ -7964,10 +8299,15 @@
       </c>
       <c r="U71" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V71" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V71" s="5" t="inlineStr"/>
+      <c r="W71" s="5" t="inlineStr"/>
     </row>
     <row r="72" ht="20" customHeight="1">
       <c r="A72" s="4" t="inlineStr">
@@ -8072,10 +8412,15 @@
       </c>
       <c r="U72" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V72" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V72" s="5" t="inlineStr"/>
+      <c r="W72" s="5" t="inlineStr"/>
     </row>
     <row r="73" ht="20" customHeight="1">
       <c r="A73" s="7" t="inlineStr">
@@ -8176,10 +8521,15 @@
       </c>
       <c r="U73" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V73" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V73" s="8" t="inlineStr">
+      <c r="W73" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -8288,10 +8638,15 @@
       </c>
       <c r="U74" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V74" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V74" s="5" t="inlineStr"/>
+      <c r="W74" s="5" t="inlineStr"/>
     </row>
     <row r="75" ht="20" customHeight="1">
       <c r="A75" s="4" t="inlineStr">
@@ -8396,10 +8751,15 @@
       </c>
       <c r="U75" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V75" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V75" s="5" t="inlineStr"/>
+      <c r="W75" s="5" t="inlineStr"/>
     </row>
     <row r="76" ht="20" customHeight="1">
       <c r="A76" s="4" t="inlineStr">
@@ -8504,10 +8864,15 @@
       </c>
       <c r="U76" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V76" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V76" s="5" t="inlineStr"/>
+      <c r="W76" s="5" t="inlineStr"/>
     </row>
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="10" t="inlineStr">
@@ -8612,10 +8977,15 @@
       </c>
       <c r="U77" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V77" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V77" s="11" t="inlineStr">
+      <c r="W77" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:12)</t>
         </is>
@@ -8720,10 +9090,15 @@
       </c>
       <c r="U78" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V78" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V78" s="8" t="inlineStr">
+      <c r="W78" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -8817,25 +9192,30 @@
       </c>
       <c r="R79" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:18</t>
         </is>
       </c>
       <c r="S79" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T79" s="6" t="inlineStr">
+        <is>
           <t>01:18</t>
         </is>
       </c>
-      <c r="T79" s="6" t="inlineStr">
-        <is>
-          <t>01:18</t>
-        </is>
-      </c>
       <c r="U79" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V79" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V79" s="5" t="inlineStr">
+      <c r="W79" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:18)</t>
         </is>
@@ -8929,25 +9309,30 @@
       </c>
       <c r="R80" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="S80" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T80" s="6" t="inlineStr">
+        <is>
           <t>02:38</t>
         </is>
       </c>
-      <c r="T80" s="6" t="inlineStr">
-        <is>
-          <t>02:38</t>
-        </is>
-      </c>
       <c r="U80" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V80" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V80" s="5" t="inlineStr">
+      <c r="W80" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (02:38)</t>
         </is>
@@ -9056,10 +9441,15 @@
       </c>
       <c r="U81" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V81" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V81" s="5" t="inlineStr"/>
+      <c r="W81" s="5" t="inlineStr"/>
     </row>
     <row r="82" ht="20" customHeight="1">
       <c r="A82" s="4" t="inlineStr">
@@ -9164,10 +9554,15 @@
       </c>
       <c r="U82" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V82" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V82" s="5" t="inlineStr"/>
+      <c r="W82" s="5" t="inlineStr"/>
     </row>
     <row r="83" ht="20" customHeight="1">
       <c r="A83" s="7" t="inlineStr">
@@ -9268,10 +9663,15 @@
       </c>
       <c r="U83" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V83" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V83" s="8" t="inlineStr">
+      <c r="W83" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -9380,10 +9780,15 @@
       </c>
       <c r="U84" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V84" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V84" s="5" t="inlineStr"/>
+      <c r="W84" s="5" t="inlineStr"/>
     </row>
     <row r="85" ht="20" customHeight="1">
       <c r="A85" s="4" t="inlineStr">
@@ -9488,10 +9893,15 @@
       </c>
       <c r="U85" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V85" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V85" s="5" t="inlineStr"/>
+      <c r="W85" s="5" t="inlineStr"/>
     </row>
     <row r="86" ht="20" customHeight="1">
       <c r="A86" s="4" t="inlineStr">
@@ -9596,10 +10006,15 @@
       </c>
       <c r="U86" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V86" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V86" s="5" t="inlineStr"/>
+      <c r="W86" s="5" t="inlineStr"/>
     </row>
     <row r="87" ht="20" customHeight="1">
       <c r="A87" s="4" t="inlineStr">
@@ -9704,10 +10119,15 @@
       </c>
       <c r="U87" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V87" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V87" s="5" t="inlineStr"/>
+      <c r="W87" s="5" t="inlineStr"/>
     </row>
     <row r="88" ht="20" customHeight="1">
       <c r="A88" s="10" t="inlineStr">
@@ -9797,25 +10217,30 @@
       </c>
       <c r="R88" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S88" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T88" s="12" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U88" s="12" t="inlineStr">
+        <is>
           <t>00:02</t>
         </is>
       </c>
-      <c r="S88" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T88" s="12" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U88" s="12" t="inlineStr">
+      <c r="V88" s="12" t="inlineStr">
         <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V88" s="11" t="inlineStr">
+      <c r="W88" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (05:43), Entrada duplicada (07:17, 07:18), Tardanza (00:02)</t>
         </is>
@@ -9924,10 +10349,15 @@
       </c>
       <c r="U89" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V89" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V89" s="5" t="inlineStr"/>
+      <c r="W89" s="5" t="inlineStr"/>
     </row>
     <row r="90" ht="20" customHeight="1">
       <c r="A90" s="4" t="inlineStr">
@@ -10017,25 +10447,30 @@
       </c>
       <c r="R90" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:17</t>
         </is>
       </c>
       <c r="S90" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T90" s="6" t="inlineStr">
+        <is>
           <t>01:17</t>
         </is>
       </c>
-      <c r="T90" s="6" t="inlineStr">
-        <is>
-          <t>01:17</t>
-        </is>
-      </c>
       <c r="U90" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V90" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V90" s="5" t="inlineStr">
+      <c r="W90" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:17)</t>
         </is>
@@ -10129,25 +10564,30 @@
       </c>
       <c r="R91" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="S91" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T91" s="6" t="inlineStr">
+        <is>
           <t>02:38</t>
         </is>
       </c>
-      <c r="T91" s="6" t="inlineStr">
-        <is>
-          <t>02:38</t>
-        </is>
-      </c>
       <c r="U91" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V91" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V91" s="5" t="inlineStr">
+      <c r="W91" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (02:38)</t>
         </is>
@@ -10256,10 +10696,15 @@
       </c>
       <c r="U92" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V92" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V92" s="5" t="inlineStr"/>
+      <c r="W92" s="5" t="inlineStr"/>
     </row>
     <row r="93" ht="20" customHeight="1">
       <c r="A93" s="4" t="inlineStr">
@@ -10364,10 +10809,15 @@
       </c>
       <c r="U93" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V93" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V93" s="5" t="inlineStr"/>
+      <c r="W93" s="5" t="inlineStr"/>
     </row>
     <row r="94" ht="20" customHeight="1">
       <c r="A94" s="7" t="inlineStr">
@@ -10468,10 +10918,15 @@
       </c>
       <c r="U94" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V94" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V94" s="8" t="inlineStr">
+      <c r="W94" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -10565,25 +11020,30 @@
       </c>
       <c r="R95" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S95" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T95" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U95" s="6" t="inlineStr">
+        <is>
           <t>00:41</t>
         </is>
       </c>
-      <c r="S95" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T95" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U95" s="6" t="inlineStr">
+      <c r="V95" s="6" t="inlineStr">
         <is>
           <t>Tardanza</t>
         </is>
       </c>
-      <c r="V95" s="5" t="inlineStr">
+      <c r="W95" s="5" t="inlineStr">
         <is>
           <t>Tardanza (00:41)</t>
         </is>
@@ -10692,10 +11152,15 @@
       </c>
       <c r="U96" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V96" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V96" s="5" t="inlineStr"/>
+      <c r="W96" s="5" t="inlineStr"/>
     </row>
     <row r="97" ht="20" customHeight="1">
       <c r="A97" s="4" t="inlineStr">
@@ -10800,10 +11265,15 @@
       </c>
       <c r="U97" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V97" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V97" s="5" t="inlineStr"/>
+      <c r="W97" s="5" t="inlineStr"/>
     </row>
     <row r="98" ht="20" customHeight="1">
       <c r="A98" s="10" t="inlineStr">
@@ -10908,10 +11378,15 @@
       </c>
       <c r="U98" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V98" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V98" s="11" t="inlineStr">
+      <c r="W98" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:15)</t>
         </is>
@@ -11016,10 +11491,15 @@
       </c>
       <c r="U99" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V99" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V99" s="8" t="inlineStr">
+      <c r="W99" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -11113,25 +11593,30 @@
       </c>
       <c r="R100" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S100" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T100" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U100" s="6" t="inlineStr">
+        <is>
           <t>03:32</t>
         </is>
       </c>
-      <c r="S100" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T100" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U100" s="6" t="inlineStr">
+      <c r="V100" s="6" t="inlineStr">
         <is>
           <t>Tardanza</t>
         </is>
       </c>
-      <c r="V100" s="5" t="inlineStr">
+      <c r="W100" s="5" t="inlineStr">
         <is>
           <t>Tardanza (03:32)</t>
         </is>
@@ -11236,10 +11721,15 @@
       </c>
       <c r="U101" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V101" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V101" s="8" t="inlineStr">
+      <c r="W101" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -11348,10 +11838,15 @@
       </c>
       <c r="U102" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V102" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V102" s="5" t="inlineStr"/>
+      <c r="W102" s="5" t="inlineStr"/>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="A103" s="4" t="inlineStr">
@@ -11456,10 +11951,15 @@
       </c>
       <c r="U103" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V103" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V103" s="5" t="inlineStr"/>
+      <c r="W103" s="5" t="inlineStr"/>
     </row>
     <row r="104" ht="20" customHeight="1">
       <c r="A104" s="7" t="inlineStr">
@@ -11560,10 +12060,15 @@
       </c>
       <c r="U104" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V104" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V104" s="8" t="inlineStr"/>
+      <c r="W104" s="8" t="inlineStr"/>
     </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="10" t="inlineStr">
@@ -11668,10 +12173,15 @@
       </c>
       <c r="U105" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V105" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V105" s="11" t="inlineStr">
+      <c r="W105" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:07)</t>
         </is>
@@ -11780,10 +12290,15 @@
       </c>
       <c r="U106" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V106" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V106" s="11" t="inlineStr">
+      <c r="W106" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (05:55)</t>
         </is>
@@ -11892,10 +12407,15 @@
       </c>
       <c r="U107" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V107" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V107" s="5" t="inlineStr"/>
+      <c r="W107" s="5" t="inlineStr"/>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="4" t="inlineStr">
@@ -12000,10 +12520,15 @@
       </c>
       <c r="U108" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V108" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V108" s="5" t="inlineStr"/>
+      <c r="W108" s="5" t="inlineStr"/>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="4" t="inlineStr">
@@ -12108,10 +12633,15 @@
       </c>
       <c r="U109" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V109" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V109" s="5" t="inlineStr"/>
+      <c r="W109" s="5" t="inlineStr"/>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="7" t="inlineStr">
@@ -12212,10 +12742,15 @@
       </c>
       <c r="U110" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V110" s="9" t="inlineStr">
+        <is>
           <t>Entrada pendiente</t>
         </is>
       </c>
-      <c r="V110" s="8" t="inlineStr">
+      <c r="W110" s="8" t="inlineStr">
         <is>
           <t>Salida sin registro de entrada previa (18:54)</t>
         </is>
@@ -12324,10 +12859,15 @@
       </c>
       <c r="U111" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V111" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V111" s="5" t="inlineStr"/>
+      <c r="W111" s="5" t="inlineStr"/>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="4" t="inlineStr">
@@ -12432,10 +12972,15 @@
       </c>
       <c r="U112" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V112" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V112" s="5" t="inlineStr"/>
+      <c r="W112" s="5" t="inlineStr"/>
     </row>
     <row r="113" ht="20" customHeight="1">
       <c r="A113" s="4" t="inlineStr">
@@ -12540,10 +13085,15 @@
       </c>
       <c r="U113" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V113" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V113" s="5" t="inlineStr"/>
+      <c r="W113" s="5" t="inlineStr"/>
     </row>
     <row r="114" ht="20" customHeight="1">
       <c r="A114" s="7" t="inlineStr">
@@ -12644,10 +13194,15 @@
       </c>
       <c r="U114" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V114" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V114" s="8" t="inlineStr">
+      <c r="W114" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -12756,10 +13311,15 @@
       </c>
       <c r="U115" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V115" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V115" s="5" t="inlineStr"/>
+      <c r="W115" s="5" t="inlineStr"/>
     </row>
     <row r="116" ht="20" customHeight="1">
       <c r="A116" s="4" t="inlineStr">
@@ -12864,10 +13424,15 @@
       </c>
       <c r="U116" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V116" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V116" s="5" t="inlineStr"/>
+      <c r="W116" s="5" t="inlineStr"/>
     </row>
     <row r="117" ht="20" customHeight="1">
       <c r="A117" s="4" t="inlineStr">
@@ -12972,10 +13537,15 @@
       </c>
       <c r="U117" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V117" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V117" s="5" t="inlineStr"/>
+      <c r="W117" s="5" t="inlineStr"/>
     </row>
     <row r="118" ht="20" customHeight="1">
       <c r="A118" s="10" t="inlineStr">
@@ -13080,10 +13650,15 @@
       </c>
       <c r="U118" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V118" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V118" s="11" t="inlineStr">
+      <c r="W118" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:12)</t>
         </is>
@@ -13188,10 +13763,15 @@
       </c>
       <c r="U119" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V119" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V119" s="8" t="inlineStr">
+      <c r="W119" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -13300,10 +13880,15 @@
       </c>
       <c r="U120" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V120" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V120" s="5" t="inlineStr"/>
+      <c r="W120" s="5" t="inlineStr"/>
     </row>
     <row r="121" ht="20" customHeight="1">
       <c r="A121" s="4" t="inlineStr">
@@ -13408,10 +13993,15 @@
       </c>
       <c r="U121" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V121" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V121" s="5" t="inlineStr"/>
+      <c r="W121" s="5" t="inlineStr"/>
     </row>
     <row r="122" ht="20" customHeight="1">
       <c r="A122" s="4" t="inlineStr">
@@ -13516,10 +14106,15 @@
       </c>
       <c r="U122" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V122" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V122" s="5" t="inlineStr"/>
+      <c r="W122" s="5" t="inlineStr"/>
     </row>
     <row r="123" ht="20" customHeight="1">
       <c r="A123" s="4" t="inlineStr">
@@ -13624,10 +14219,15 @@
       </c>
       <c r="U123" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V123" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V123" s="5" t="inlineStr"/>
+      <c r="W123" s="5" t="inlineStr"/>
     </row>
     <row r="124" ht="20" customHeight="1">
       <c r="A124" s="7" t="inlineStr">
@@ -13728,10 +14328,15 @@
       </c>
       <c r="U124" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V124" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V124" s="8" t="inlineStr">
+      <c r="W124" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -13840,10 +14445,15 @@
       </c>
       <c r="U125" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V125" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V125" s="5" t="inlineStr"/>
+      <c r="W125" s="5" t="inlineStr"/>
     </row>
     <row r="126" ht="20" customHeight="1">
       <c r="A126" s="4" t="inlineStr">
@@ -13948,10 +14558,15 @@
       </c>
       <c r="U126" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V126" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V126" s="5" t="inlineStr"/>
+      <c r="W126" s="5" t="inlineStr"/>
     </row>
     <row r="127" ht="20" customHeight="1">
       <c r="A127" s="4" t="inlineStr">
@@ -14041,25 +14656,30 @@
       </c>
       <c r="R127" s="6" t="inlineStr">
         <is>
+          <t>01:13</t>
+        </is>
+      </c>
+      <c r="S127" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T127" s="6" t="inlineStr">
+        <is>
+          <t>01:13</t>
+        </is>
+      </c>
+      <c r="U127" s="6" t="inlineStr">
+        <is>
           <t>00:33</t>
         </is>
       </c>
-      <c r="S127" s="6" t="inlineStr">
-        <is>
-          <t>01:13</t>
-        </is>
-      </c>
-      <c r="T127" s="6" t="inlineStr">
-        <is>
-          <t>01:13</t>
-        </is>
-      </c>
-      <c r="U127" s="6" t="inlineStr">
+      <c r="V127" s="6" t="inlineStr">
         <is>
           <t>Exceso de Jornada/Tardanza</t>
         </is>
       </c>
-      <c r="V127" s="5" t="inlineStr">
+      <c r="W127" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:13), Tardanza (00:33)</t>
         </is>
@@ -14168,10 +14788,15 @@
       </c>
       <c r="U128" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V128" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V128" s="11" t="inlineStr">
+      <c r="W128" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:09)</t>
         </is>
@@ -14276,10 +14901,15 @@
       </c>
       <c r="U129" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V129" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V129" s="8" t="inlineStr">
+      <c r="W129" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -14388,10 +15018,15 @@
       </c>
       <c r="U130" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V130" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V130" s="5" t="inlineStr"/>
+      <c r="W130" s="5" t="inlineStr"/>
     </row>
     <row r="131" ht="20" customHeight="1">
       <c r="A131" s="4" t="inlineStr">
@@ -14496,10 +15131,15 @@
       </c>
       <c r="U131" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V131" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V131" s="5" t="inlineStr"/>
+      <c r="W131" s="5" t="inlineStr"/>
     </row>
     <row r="132" ht="20" customHeight="1">
       <c r="A132" s="4" t="inlineStr">
@@ -14604,10 +15244,15 @@
       </c>
       <c r="U132" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V132" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V132" s="5" t="inlineStr"/>
+      <c r="W132" s="5" t="inlineStr"/>
     </row>
     <row r="133" ht="20" customHeight="1">
       <c r="A133" s="4" t="inlineStr">
@@ -14712,10 +15357,15 @@
       </c>
       <c r="U133" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V133" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V133" s="5" t="inlineStr"/>
+      <c r="W133" s="5" t="inlineStr"/>
     </row>
     <row r="134" ht="20" customHeight="1">
       <c r="A134" s="4" t="inlineStr">
@@ -14820,10 +15470,15 @@
       </c>
       <c r="U134" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V134" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V134" s="5" t="inlineStr"/>
+      <c r="W134" s="5" t="inlineStr"/>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="10" t="inlineStr">
@@ -14928,10 +15583,15 @@
       </c>
       <c r="U135" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V135" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V135" s="11" t="inlineStr">
+      <c r="W135" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (07:55)</t>
         </is>
@@ -15040,10 +15700,15 @@
       </c>
       <c r="U136" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V136" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V136" s="11" t="inlineStr">
+      <c r="W136" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:00)</t>
         </is>
@@ -15152,10 +15817,15 @@
       </c>
       <c r="U137" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V137" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V137" s="5" t="inlineStr"/>
+      <c r="W137" s="5" t="inlineStr"/>
     </row>
     <row r="138" ht="20" customHeight="1">
       <c r="A138" s="4" t="inlineStr">
@@ -15260,10 +15930,15 @@
       </c>
       <c r="U138" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V138" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V138" s="5" t="inlineStr"/>
+      <c r="W138" s="5" t="inlineStr"/>
     </row>
     <row r="139" ht="20" customHeight="1">
       <c r="A139" s="4" t="inlineStr">
@@ -15368,10 +16043,15 @@
       </c>
       <c r="U139" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V139" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V139" s="5" t="inlineStr"/>
+      <c r="W139" s="5" t="inlineStr"/>
     </row>
     <row r="140" ht="20" customHeight="1">
       <c r="A140" s="4" t="inlineStr">
@@ -15476,10 +16156,15 @@
       </c>
       <c r="U140" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V140" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V140" s="5" t="inlineStr"/>
+      <c r="W140" s="5" t="inlineStr"/>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="4" t="inlineStr">
@@ -15584,10 +16269,15 @@
       </c>
       <c r="U141" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V141" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V141" s="5" t="inlineStr"/>
+      <c r="W141" s="5" t="inlineStr"/>
     </row>
     <row r="142" ht="20" customHeight="1">
       <c r="A142" s="4" t="inlineStr">
@@ -15692,10 +16382,15 @@
       </c>
       <c r="U142" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V142" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V142" s="5" t="inlineStr"/>
+      <c r="W142" s="5" t="inlineStr"/>
     </row>
     <row r="143" ht="20" customHeight="1">
       <c r="A143" s="4" t="inlineStr">
@@ -15800,10 +16495,15 @@
       </c>
       <c r="U143" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V143" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V143" s="5" t="inlineStr"/>
+      <c r="W143" s="5" t="inlineStr"/>
     </row>
     <row r="144" ht="20" customHeight="1">
       <c r="A144" s="7" t="inlineStr">
@@ -15889,25 +16589,30 @@
       </c>
       <c r="R144" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S144" s="9" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T144" s="9" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U144" s="9" t="inlineStr">
+        <is>
           <t>00:29</t>
         </is>
       </c>
-      <c r="S144" s="9" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T144" s="9" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U144" s="9" t="inlineStr">
+      <c r="V144" s="9" t="inlineStr">
         <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V144" s="8" t="inlineStr">
+      <c r="W144" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida, Tardanza (00:29)</t>
         </is>
@@ -16016,10 +16721,15 @@
       </c>
       <c r="U145" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V145" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V145" s="5" t="inlineStr">
+      <c r="W145" s="5" t="inlineStr">
         <is>
           <t>Entrada duplicada (06:36, 06:37)</t>
         </is>
@@ -16113,25 +16823,30 @@
       </c>
       <c r="R146" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>01:23</t>
         </is>
       </c>
       <c r="S146" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T146" s="6" t="inlineStr">
+        <is>
           <t>01:23</t>
         </is>
       </c>
-      <c r="T146" s="6" t="inlineStr">
-        <is>
-          <t>01:23</t>
-        </is>
-      </c>
       <c r="U146" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V146" s="6" t="inlineStr">
+        <is>
           <t>Exceso de Jornada</t>
         </is>
       </c>
-      <c r="V146" s="5" t="inlineStr">
+      <c r="W146" s="5" t="inlineStr">
         <is>
           <t>Exceso de Jornada (01:23)</t>
         </is>
@@ -16236,10 +16951,15 @@
       </c>
       <c r="U147" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V147" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V147" s="8" t="inlineStr">
+      <c r="W147" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -16348,10 +17068,15 @@
       </c>
       <c r="U148" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V148" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V148" s="5" t="inlineStr"/>
+      <c r="W148" s="5" t="inlineStr"/>
     </row>
     <row r="149" ht="20" customHeight="1">
       <c r="A149" s="4" t="inlineStr">
@@ -16456,10 +17181,15 @@
       </c>
       <c r="U149" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V149" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V149" s="5" t="inlineStr"/>
+      <c r="W149" s="5" t="inlineStr"/>
     </row>
     <row r="150" ht="20" customHeight="1">
       <c r="A150" s="4" t="inlineStr">
@@ -16564,10 +17294,15 @@
       </c>
       <c r="U150" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V150" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V150" s="5" t="inlineStr"/>
+      <c r="W150" s="5" t="inlineStr"/>
     </row>
     <row r="151" ht="20" customHeight="1">
       <c r="A151" s="4" t="inlineStr">
@@ -16657,25 +17392,30 @@
       </c>
       <c r="R151" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S151" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T151" s="6" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U151" s="6" t="inlineStr">
+        <is>
           <t>00:39</t>
         </is>
       </c>
-      <c r="S151" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T151" s="6" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U151" s="6" t="inlineStr">
+      <c r="V151" s="6" t="inlineStr">
         <is>
           <t>Tardanza</t>
         </is>
       </c>
-      <c r="V151" s="5" t="inlineStr">
+      <c r="W151" s="5" t="inlineStr">
         <is>
           <t>Tardanza (00:39)</t>
         </is>
@@ -16784,10 +17524,15 @@
       </c>
       <c r="U152" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V152" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V152" s="5" t="inlineStr"/>
+      <c r="W152" s="5" t="inlineStr"/>
     </row>
     <row r="153" ht="20" customHeight="1">
       <c r="A153" s="7" t="inlineStr">
@@ -16888,10 +17633,15 @@
       </c>
       <c r="U153" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V153" s="9" t="inlineStr">
+        <is>
           <t>Entrada pendiente</t>
         </is>
       </c>
-      <c r="V153" s="8" t="inlineStr">
+      <c r="W153" s="8" t="inlineStr">
         <is>
           <t>Salida sin registro de entrada previa (19:06)</t>
         </is>
@@ -17000,10 +17750,15 @@
       </c>
       <c r="U154" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V154" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V154" s="5" t="inlineStr"/>
+      <c r="W154" s="5" t="inlineStr"/>
     </row>
     <row r="155" ht="20" customHeight="1">
       <c r="A155" s="7" t="inlineStr">
@@ -17104,10 +17859,15 @@
       </c>
       <c r="U155" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V155" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V155" s="8" t="inlineStr">
+      <c r="W155" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -17197,25 +17957,30 @@
       </c>
       <c r="R156" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="S156" s="9" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="T156" s="9" t="inlineStr">
+        <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="U156" s="9" t="inlineStr">
+        <is>
           <t>00:32</t>
         </is>
       </c>
-      <c r="S156" s="9" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="T156" s="9" t="inlineStr">
-        <is>
-          <t>00:00</t>
-        </is>
-      </c>
-      <c r="U156" s="9" t="inlineStr">
+      <c r="V156" s="9" t="inlineStr">
         <is>
           <t>Salida pendiente/Tardanza</t>
         </is>
       </c>
-      <c r="V156" s="8" t="inlineStr">
+      <c r="W156" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida, Tardanza (00:32)</t>
         </is>
@@ -17324,10 +18089,15 @@
       </c>
       <c r="U157" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V157" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V157" s="5" t="inlineStr"/>
+      <c r="W157" s="5" t="inlineStr"/>
     </row>
     <row r="158" ht="20" customHeight="1">
       <c r="A158" s="4" t="inlineStr">
@@ -17432,10 +18202,15 @@
       </c>
       <c r="U158" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V158" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V158" s="5" t="inlineStr"/>
+      <c r="W158" s="5" t="inlineStr"/>
     </row>
     <row r="159" ht="20" customHeight="1">
       <c r="A159" s="4" t="inlineStr">
@@ -17540,10 +18315,15 @@
       </c>
       <c r="U159" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V159" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V159" s="5" t="inlineStr"/>
+      <c r="W159" s="5" t="inlineStr"/>
     </row>
     <row r="160" ht="20" customHeight="1">
       <c r="A160" s="10" t="inlineStr">
@@ -17648,10 +18428,15 @@
       </c>
       <c r="U160" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V160" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V160" s="11" t="inlineStr">
+      <c r="W160" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (05:51)</t>
         </is>
@@ -17760,10 +18545,15 @@
       </c>
       <c r="U161" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V161" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V161" s="5" t="inlineStr"/>
+      <c r="W161" s="5" t="inlineStr"/>
     </row>
     <row r="162" ht="20" customHeight="1">
       <c r="A162" s="4" t="inlineStr">
@@ -17868,10 +18658,15 @@
       </c>
       <c r="U162" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V162" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V162" s="5" t="inlineStr"/>
+      <c r="W162" s="5" t="inlineStr"/>
     </row>
     <row r="163" ht="20" customHeight="1">
       <c r="A163" s="4" t="inlineStr">
@@ -17976,10 +18771,15 @@
       </c>
       <c r="U163" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V163" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V163" s="5" t="inlineStr"/>
+      <c r="W163" s="5" t="inlineStr"/>
     </row>
     <row r="164" ht="20" customHeight="1">
       <c r="A164" s="4" t="inlineStr">
@@ -18084,10 +18884,15 @@
       </c>
       <c r="U164" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V164" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V164" s="5" t="inlineStr"/>
+      <c r="W164" s="5" t="inlineStr"/>
     </row>
     <row r="165" ht="20" customHeight="1">
       <c r="A165" s="4" t="inlineStr">
@@ -18192,10 +18997,15 @@
       </c>
       <c r="U165" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V165" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V165" s="5" t="inlineStr"/>
+      <c r="W165" s="5" t="inlineStr"/>
     </row>
     <row r="166" ht="20" customHeight="1">
       <c r="A166" s="7" t="inlineStr">
@@ -18296,10 +19106,15 @@
       </c>
       <c r="U166" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V166" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V166" s="8" t="inlineStr">
+      <c r="W166" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -18408,10 +19223,15 @@
       </c>
       <c r="U167" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V167" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V167" s="5" t="inlineStr"/>
+      <c r="W167" s="5" t="inlineStr"/>
     </row>
     <row r="168" ht="20" customHeight="1">
       <c r="A168" s="4" t="inlineStr">
@@ -18516,10 +19336,15 @@
       </c>
       <c r="U168" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V168" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V168" s="5" t="inlineStr"/>
+      <c r="W168" s="5" t="inlineStr"/>
     </row>
     <row r="169" ht="20" customHeight="1">
       <c r="A169" s="4" t="inlineStr">
@@ -18614,7 +19439,7 @@
       </c>
       <c r="S169" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:43</t>
         </is>
       </c>
       <c r="T169" s="6" t="inlineStr">
@@ -18624,10 +19449,15 @@
       </c>
       <c r="U169" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V169" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V169" s="5" t="inlineStr">
+      <c r="W169" s="5" t="inlineStr">
         <is>
           <t>Horas extras (02:43)</t>
         </is>
@@ -18726,7 +19556,7 @@
       </c>
       <c r="S170" s="6" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="T170" s="6" t="inlineStr">
@@ -18736,10 +19566,15 @@
       </c>
       <c r="U170" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V170" s="6" t="inlineStr">
+        <is>
           <t>Horas extras</t>
         </is>
       </c>
-      <c r="V170" s="5" t="inlineStr">
+      <c r="W170" s="5" t="inlineStr">
         <is>
           <t>Horas extras (02:00)</t>
         </is>
@@ -18844,10 +19679,15 @@
       </c>
       <c r="U171" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V171" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V171" s="8" t="inlineStr">
+      <c r="W171" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -18956,10 +19796,15 @@
       </c>
       <c r="U172" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V172" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V172" s="5" t="inlineStr"/>
+      <c r="W172" s="5" t="inlineStr"/>
     </row>
     <row r="173" ht="20" customHeight="1">
       <c r="A173" s="4" t="inlineStr">
@@ -19064,10 +19909,15 @@
       </c>
       <c r="U173" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V173" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V173" s="5" t="inlineStr"/>
+      <c r="W173" s="5" t="inlineStr"/>
     </row>
     <row r="174" ht="20" customHeight="1">
       <c r="A174" s="4" t="inlineStr">
@@ -19172,10 +20022,15 @@
       </c>
       <c r="U174" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V174" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V174" s="5" t="inlineStr"/>
+      <c r="W174" s="5" t="inlineStr"/>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="4" t="inlineStr">
@@ -19280,10 +20135,15 @@
       </c>
       <c r="U175" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V175" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V175" s="5" t="inlineStr"/>
+      <c r="W175" s="5" t="inlineStr"/>
     </row>
     <row r="176" ht="20" customHeight="1">
       <c r="A176" s="7" t="inlineStr">
@@ -19384,10 +20244,15 @@
       </c>
       <c r="U176" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V176" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V176" s="8" t="inlineStr">
+      <c r="W176" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -19496,10 +20361,15 @@
       </c>
       <c r="U177" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V177" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V177" s="5" t="inlineStr"/>
+      <c r="W177" s="5" t="inlineStr"/>
     </row>
     <row r="178" ht="20" customHeight="1">
       <c r="A178" s="4" t="inlineStr">
@@ -19604,10 +20474,15 @@
       </c>
       <c r="U178" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V178" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V178" s="5" t="inlineStr"/>
+      <c r="W178" s="5" t="inlineStr"/>
     </row>
     <row r="179" ht="20" customHeight="1">
       <c r="A179" s="4" t="inlineStr">
@@ -19712,10 +20587,15 @@
       </c>
       <c r="U179" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V179" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V179" s="5" t="inlineStr"/>
+      <c r="W179" s="5" t="inlineStr"/>
     </row>
     <row r="180" ht="20" customHeight="1">
       <c r="A180" s="10" t="inlineStr">
@@ -19820,10 +20700,15 @@
       </c>
       <c r="U180" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V180" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V180" s="11" t="inlineStr">
+      <c r="W180" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:26)</t>
         </is>
@@ -19928,10 +20813,15 @@
       </c>
       <c r="U181" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V181" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V181" s="8" t="inlineStr">
+      <c r="W181" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -20040,10 +20930,15 @@
       </c>
       <c r="U182" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V182" s="6" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="V182" s="5" t="inlineStr"/>
+      <c r="W182" s="5" t="inlineStr"/>
     </row>
     <row r="183" ht="20" customHeight="1">
       <c r="A183" s="4" t="inlineStr">
@@ -20148,10 +21043,15 @@
       </c>
       <c r="U183" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V183" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V183" s="5" t="inlineStr"/>
+      <c r="W183" s="5" t="inlineStr"/>
     </row>
     <row r="184" ht="20" customHeight="1">
       <c r="A184" s="4" t="inlineStr">
@@ -20256,10 +21156,15 @@
       </c>
       <c r="U184" s="6" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V184" s="6" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V184" s="5" t="inlineStr"/>
+      <c r="W184" s="5" t="inlineStr"/>
     </row>
     <row r="185" ht="20" customHeight="1">
       <c r="A185" s="10" t="inlineStr">
@@ -20364,10 +21269,15 @@
       </c>
       <c r="U185" s="12" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V185" s="12" t="inlineStr">
+        <is>
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="V185" s="11" t="inlineStr">
+      <c r="W185" s="11" t="inlineStr">
         <is>
           <t>Jornada parcial (Medio día) (06:25)</t>
         </is>
@@ -20472,10 +21382,15 @@
       </c>
       <c r="U186" s="9" t="inlineStr">
         <is>
+          <t>00:00</t>
+        </is>
+      </c>
+      <c r="V186" s="9" t="inlineStr">
+        <is>
           <t>Salida pendiente</t>
         </is>
       </c>
-      <c r="V186" s="8" t="inlineStr">
+      <c r="W186" s="8" t="inlineStr">
         <is>
           <t>Falta marcación de salida</t>
         </is>
@@ -20483,7 +21398,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="A2:W2"/>
     <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
style: Executive pastel color palette with high-contrast text for calculation column headers
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -46,10 +46,22 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00833C0C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -76,14 +88,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002F5597"/>
-        <bgColor rgb="002F5597"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C65911"/>
-        <bgColor rgb="00C65911"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -130,37 +136,37 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>

</xml_diff>

<commit_message>
style: Extended Teal header fill (#317F96) from column Q to W as shown in user's image
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -663,17 +663,17 @@
           <t>Total de Horas Adicionales</t>
         </is>
       </c>
-      <c r="U4" s="3" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>Tardanza</t>
         </is>
       </c>
-      <c r="V4" s="3" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>Tipo Registro</t>
         </is>
       </c>
-      <c r="W4" s="3" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>Observación / Incidencias</t>
         </is>

</xml_diff>

<commit_message>
style: Applied Teal header fill (#317F96) strictly to columns Q to U (Horas de Turno to Tardanza) as requested in latest screenshot
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -668,12 +668,12 @@
           <t>Tardanza</t>
         </is>
       </c>
-      <c r="V4" s="4" t="inlineStr">
+      <c r="V4" s="3" t="inlineStr">
         <is>
           <t>Tipo Registro</t>
         </is>
       </c>
-      <c r="W4" s="4" t="inlineStr">
+      <c r="W4" s="3" t="inlineStr">
         <is>
           <t>Observación / Incidencias</t>
         </is>

</xml_diff>

<commit_message>
fix: Calculate worked hours and excess shift using real entry swipe timestamp instead of artificial snapping to 07:00/19:00
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -866,7 +866,7 @@
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>12:26</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:43</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:43</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
@@ -1004,10 +1004,14 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W7" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:43)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1318,7 +1322,7 @@
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>12:11</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
@@ -1431,12 +1435,12 @@
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="S11" s="7" t="inlineStr">
@@ -1446,7 +1450,7 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -1456,10 +1460,14 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W11" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:30)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1774,7 +1782,7 @@
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
@@ -1887,7 +1895,7 @@
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
@@ -2000,7 +2008,7 @@
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>10:23</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
@@ -2113,12 +2121,12 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>13:56</t>
+          <t>14:09</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>01:56</t>
+          <t>02:09</t>
         </is>
       </c>
       <c r="S17" s="7" t="inlineStr">
@@ -2128,7 +2136,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>01:56</t>
+          <t>02:09</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
@@ -2143,7 +2151,7 @@
       </c>
       <c r="W17" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:56)</t>
+          <t>Exceso de Jornada (02:09)</t>
         </is>
       </c>
     </row>
@@ -2230,12 +2238,12 @@
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="S18" s="7" t="inlineStr">
@@ -2245,7 +2253,7 @@
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="U18" s="7" t="inlineStr">
@@ -2255,10 +2263,14 @@
       </c>
       <c r="V18" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W18" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W18" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:31)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -2343,7 +2355,7 @@
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
@@ -2456,7 +2468,7 @@
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
@@ -2682,7 +2694,7 @@
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
@@ -2912,7 +2924,7 @@
       </c>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
@@ -3025,7 +3037,7 @@
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>12:26</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
@@ -3138,7 +3150,7 @@
       </c>
       <c r="Q26" s="10" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="R26" s="10" t="inlineStr">
@@ -3372,12 +3384,12 @@
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:46</t>
         </is>
       </c>
       <c r="S28" s="7" t="inlineStr">
@@ -3387,7 +3399,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:46</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
@@ -3397,12 +3409,12 @@
       </c>
       <c r="V28" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="W28" s="6" t="inlineStr">
         <is>
-          <t>Entrada duplicada (18:17)</t>
+          <t>Exceso de Jornada (00:46), Entrada duplicada (18:17)</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3501,7 @@
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:20</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
@@ -3519,7 +3531,7 @@
       </c>
       <c r="W29" s="6" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:02)</t>
+          <t>Jornada parcial (Medio día) (06:20)</t>
         </is>
       </c>
     </row>
@@ -3606,12 +3618,12 @@
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:34</t>
         </is>
       </c>
       <c r="S30" s="7" t="inlineStr">
@@ -3621,7 +3633,7 @@
       </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:34</t>
         </is>
       </c>
       <c r="U30" s="7" t="inlineStr">
@@ -3631,10 +3643,14 @@
       </c>
       <c r="V30" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W30" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W30" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:34)</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -3719,7 +3735,7 @@
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
@@ -3832,7 +3848,7 @@
       </c>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
@@ -3945,7 +3961,7 @@
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
@@ -4058,7 +4074,7 @@
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="R34" s="7" t="inlineStr">
@@ -4171,7 +4187,7 @@
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr">
@@ -4284,7 +4300,7 @@
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>12:16</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
@@ -4623,12 +4639,12 @@
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:34</t>
         </is>
       </c>
       <c r="S39" s="7" t="inlineStr">
@@ -4638,7 +4654,7 @@
       </c>
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>04:34</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
@@ -4653,7 +4669,7 @@
       </c>
       <c r="W39" s="6" t="inlineStr">
         <is>
-          <t>Horas extras (04:00)</t>
+          <t>Horas extras (04:00), Exceso de Jornada (00:34)</t>
         </is>
       </c>
     </row>
@@ -4974,7 +4990,7 @@
       </c>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
@@ -5317,12 +5333,12 @@
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>12:12</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="S45" s="7" t="inlineStr">
@@ -5332,7 +5348,7 @@
       </c>
       <c r="T45" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
@@ -5342,10 +5358,14 @@
       </c>
       <c r="V45" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W45" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W45" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:30)</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -5430,7 +5450,7 @@
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
@@ -5656,12 +5676,12 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:56</t>
         </is>
       </c>
       <c r="S48" s="7" t="inlineStr">
@@ -5671,7 +5691,7 @@
       </c>
       <c r="T48" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:56</t>
         </is>
       </c>
       <c r="U48" s="7" t="inlineStr">
@@ -5681,10 +5701,14 @@
       </c>
       <c r="V48" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W48" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W48" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:56)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -6112,12 +6136,12 @@
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:44</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:44</t>
         </is>
       </c>
       <c r="S52" s="7" t="inlineStr">
@@ -6127,7 +6151,7 @@
       </c>
       <c r="T52" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:44</t>
         </is>
       </c>
       <c r="U52" s="7" t="inlineStr">
@@ -6137,10 +6161,14 @@
       </c>
       <c r="V52" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W52" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W52" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:44)</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -6225,12 +6253,12 @@
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>12:09</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="S53" s="7" t="inlineStr">
@@ -6240,7 +6268,7 @@
       </c>
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
@@ -6250,10 +6278,14 @@
       </c>
       <c r="V53" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W53" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W53" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:31)</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
@@ -6451,12 +6483,12 @@
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="S55" s="7" t="inlineStr">
@@ -6466,7 +6498,7 @@
       </c>
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
@@ -6476,10 +6508,14 @@
       </c>
       <c r="V55" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W55" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W55" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:31)</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
@@ -6677,7 +6713,7 @@
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
@@ -6790,7 +6826,7 @@
       </c>
       <c r="Q58" s="7" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R58" s="7" t="inlineStr">
@@ -6903,12 +6939,12 @@
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>02:42</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="S59" s="7" t="inlineStr">
@@ -6918,7 +6954,7 @@
       </c>
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>02:42</t>
+          <t>03:02</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
@@ -6933,7 +6969,7 @@
       </c>
       <c r="W59" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (02:42), Entrada duplicada (06:40)</t>
+          <t>Exceso de Jornada (03:02), Entrada duplicada (06:40)</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7056,7 @@
       </c>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
@@ -7137,12 +7173,12 @@
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:43</t>
         </is>
       </c>
       <c r="S61" s="7" t="inlineStr">
@@ -7152,7 +7188,7 @@
       </c>
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:43</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
@@ -7167,7 +7203,7 @@
       </c>
       <c r="W61" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (00:30)</t>
+          <t>Exceso de Jornada (00:43)</t>
         </is>
       </c>
     </row>
@@ -8057,7 +8093,7 @@
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="R69" s="7" t="inlineStr">
@@ -8170,7 +8206,7 @@
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
@@ -8283,7 +8319,7 @@
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
@@ -8509,7 +8545,7 @@
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="R73" s="7" t="inlineStr">
@@ -8622,7 +8658,7 @@
       </c>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>10:20</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
@@ -8735,7 +8771,7 @@
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
@@ -9078,12 +9114,12 @@
       </c>
       <c r="Q78" s="7" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:34</t>
         </is>
       </c>
       <c r="R78" s="7" t="inlineStr">
         <is>
-          <t>01:18</t>
+          <t>01:34</t>
         </is>
       </c>
       <c r="S78" s="7" t="inlineStr">
@@ -9093,7 +9129,7 @@
       </c>
       <c r="T78" s="7" t="inlineStr">
         <is>
-          <t>01:18</t>
+          <t>01:34</t>
         </is>
       </c>
       <c r="U78" s="7" t="inlineStr">
@@ -9108,7 +9144,7 @@
       </c>
       <c r="W78" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:18)</t>
+          <t>Exceso de Jornada (01:34)</t>
         </is>
       </c>
     </row>
@@ -9195,12 +9231,12 @@
       </c>
       <c r="Q79" s="7" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="R79" s="7" t="inlineStr">
         <is>
-          <t>02:38</t>
+          <t>02:59</t>
         </is>
       </c>
       <c r="S79" s="7" t="inlineStr">
@@ -9210,7 +9246,7 @@
       </c>
       <c r="T79" s="7" t="inlineStr">
         <is>
-          <t>02:38</t>
+          <t>02:59</t>
         </is>
       </c>
       <c r="U79" s="7" t="inlineStr">
@@ -9225,7 +9261,7 @@
       </c>
       <c r="W79" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (02:38)</t>
+          <t>Exceso de Jornada (02:59)</t>
         </is>
       </c>
     </row>
@@ -9312,7 +9348,7 @@
       </c>
       <c r="Q80" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="R80" s="7" t="inlineStr">
@@ -9425,7 +9461,7 @@
       </c>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:16</t>
         </is>
       </c>
       <c r="R81" s="7" t="inlineStr">
@@ -9651,7 +9687,7 @@
       </c>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R83" s="7" t="inlineStr">
@@ -9764,7 +9800,7 @@
       </c>
       <c r="Q84" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R84" s="7" t="inlineStr">
@@ -9877,7 +9913,7 @@
       </c>
       <c r="Q85" s="7" t="inlineStr">
         <is>
-          <t>12:06</t>
+          <t>12:16</t>
         </is>
       </c>
       <c r="R85" s="7" t="inlineStr">
@@ -9990,7 +10026,7 @@
       </c>
       <c r="Q86" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R86" s="7" t="inlineStr">
@@ -10220,7 +10256,7 @@
       </c>
       <c r="Q88" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="R88" s="7" t="inlineStr">
@@ -10333,12 +10369,12 @@
       </c>
       <c r="Q89" s="7" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:29</t>
         </is>
       </c>
       <c r="R89" s="7" t="inlineStr">
         <is>
-          <t>01:17</t>
+          <t>01:29</t>
         </is>
       </c>
       <c r="S89" s="7" t="inlineStr">
@@ -10348,7 +10384,7 @@
       </c>
       <c r="T89" s="7" t="inlineStr">
         <is>
-          <t>01:17</t>
+          <t>01:29</t>
         </is>
       </c>
       <c r="U89" s="7" t="inlineStr">
@@ -10363,7 +10399,7 @@
       </c>
       <c r="W89" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:17)</t>
+          <t>Exceso de Jornada (01:29)</t>
         </is>
       </c>
     </row>
@@ -10450,12 +10486,12 @@
       </c>
       <c r="Q90" s="7" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="R90" s="7" t="inlineStr">
         <is>
-          <t>02:38</t>
+          <t>02:56</t>
         </is>
       </c>
       <c r="S90" s="7" t="inlineStr">
@@ -10465,7 +10501,7 @@
       </c>
       <c r="T90" s="7" t="inlineStr">
         <is>
-          <t>02:38</t>
+          <t>02:56</t>
         </is>
       </c>
       <c r="U90" s="7" t="inlineStr">
@@ -10480,7 +10516,7 @@
       </c>
       <c r="W90" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (02:38)</t>
+          <t>Exceso de Jornada (02:56)</t>
         </is>
       </c>
     </row>
@@ -10567,7 +10603,7 @@
       </c>
       <c r="Q91" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="R91" s="7" t="inlineStr">
@@ -10680,7 +10716,7 @@
       </c>
       <c r="Q92" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="R92" s="7" t="inlineStr">
@@ -11023,7 +11059,7 @@
       </c>
       <c r="Q95" s="7" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>10:27</t>
         </is>
       </c>
       <c r="R95" s="7" t="inlineStr">
@@ -11136,7 +11172,7 @@
       </c>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
@@ -11822,7 +11858,7 @@
       </c>
       <c r="Q102" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:16</t>
         </is>
       </c>
       <c r="R102" s="7" t="inlineStr">
@@ -12161,7 +12197,7 @@
       </c>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>05:55</t>
+          <t>06:07</t>
         </is>
       </c>
       <c r="R105" s="7" t="inlineStr">
@@ -12191,7 +12227,7 @@
       </c>
       <c r="W105" s="6" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (05:55)</t>
+          <t>Jornada parcial (Medio día) (06:07)</t>
         </is>
       </c>
     </row>
@@ -12278,7 +12314,7 @@
       </c>
       <c r="Q106" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="R106" s="7" t="inlineStr">
@@ -12391,7 +12427,7 @@
       </c>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="R107" s="7" t="inlineStr">
@@ -12504,7 +12540,7 @@
       </c>
       <c r="Q108" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="R108" s="7" t="inlineStr">
@@ -12730,7 +12766,7 @@
       </c>
       <c r="Q110" s="7" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R110" s="7" t="inlineStr">
@@ -12843,7 +12879,7 @@
       </c>
       <c r="Q111" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>12:16</t>
         </is>
       </c>
       <c r="R111" s="7" t="inlineStr">
@@ -12956,7 +12992,7 @@
       </c>
       <c r="Q112" s="7" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R112" s="7" t="inlineStr">
@@ -13182,7 +13218,7 @@
       </c>
       <c r="Q114" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="R114" s="7" t="inlineStr">
@@ -13295,7 +13331,7 @@
       </c>
       <c r="Q115" s="7" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="R115" s="7" t="inlineStr">
@@ -13408,7 +13444,7 @@
       </c>
       <c r="Q116" s="7" t="inlineStr">
         <is>
-          <t>14:01</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="R116" s="7" t="inlineStr">
@@ -13751,7 +13787,7 @@
       </c>
       <c r="Q119" s="7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="R119" s="7" t="inlineStr">
@@ -13864,7 +13900,7 @@
       </c>
       <c r="Q120" s="7" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>10:31</t>
         </is>
       </c>
       <c r="R120" s="7" t="inlineStr">
@@ -13977,7 +14013,7 @@
       </c>
       <c r="Q121" s="7" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="R121" s="7" t="inlineStr">
@@ -14090,7 +14126,7 @@
       </c>
       <c r="Q122" s="7" t="inlineStr">
         <is>
-          <t>11:59</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="R122" s="7" t="inlineStr">
@@ -14316,7 +14352,7 @@
       </c>
       <c r="Q124" s="7" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R124" s="7" t="inlineStr">
@@ -14429,7 +14465,7 @@
       </c>
       <c r="Q125" s="7" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>10:22</t>
         </is>
       </c>
       <c r="R125" s="7" t="inlineStr">
@@ -14889,7 +14925,7 @@
       </c>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
@@ -15115,7 +15151,7 @@
       </c>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -15228,7 +15264,7 @@
       </c>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
@@ -15341,7 +15377,7 @@
       </c>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>10:05</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
@@ -15454,7 +15490,7 @@
       </c>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
@@ -15482,11 +15518,7 @@
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="W134" s="6" t="inlineStr">
-        <is>
-          <t>Jornada parcial (Medio día) (07:55)</t>
-        </is>
-      </c>
+      <c r="W134" s="6" t="inlineStr"/>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
@@ -15571,7 +15603,7 @@
       </c>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>06:18</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
@@ -15601,7 +15633,7 @@
       </c>
       <c r="W135" s="6" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:00)</t>
+          <t>Jornada parcial (Medio día) (06:18)</t>
         </is>
       </c>
     </row>
@@ -15688,7 +15720,7 @@
       </c>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
@@ -15801,7 +15833,7 @@
       </c>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
@@ -15914,7 +15946,7 @@
       </c>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
@@ -16027,7 +16059,7 @@
       </c>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:59</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
@@ -16140,12 +16172,12 @@
       </c>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:32</t>
         </is>
       </c>
       <c r="S140" s="7" t="inlineStr">
@@ -16155,7 +16187,7 @@
       </c>
       <c r="T140" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:32</t>
         </is>
       </c>
       <c r="U140" s="7" t="inlineStr">
@@ -16165,10 +16197,14 @@
       </c>
       <c r="V140" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W140" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W140" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:32)</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
@@ -16253,7 +16289,7 @@
       </c>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
@@ -16366,7 +16402,7 @@
       </c>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
@@ -16592,12 +16628,12 @@
       </c>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:38</t>
         </is>
       </c>
       <c r="S144" s="7" t="inlineStr">
@@ -16607,7 +16643,7 @@
       </c>
       <c r="T144" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:38</t>
         </is>
       </c>
       <c r="U144" s="7" t="inlineStr">
@@ -16617,12 +16653,12 @@
       </c>
       <c r="V144" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="W144" s="6" t="inlineStr">
         <is>
-          <t>Entrada duplicada (06:36, 06:37)</t>
+          <t>Exceso de Jornada (00:38), Entrada duplicada (06:36, 06:37)</t>
         </is>
       </c>
     </row>
@@ -16709,12 +16745,12 @@
       </c>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:44</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>01:23</t>
+          <t>01:44</t>
         </is>
       </c>
       <c r="S145" s="7" t="inlineStr">
@@ -16724,7 +16760,7 @@
       </c>
       <c r="T145" s="7" t="inlineStr">
         <is>
-          <t>01:23</t>
+          <t>01:44</t>
         </is>
       </c>
       <c r="U145" s="7" t="inlineStr">
@@ -16739,7 +16775,7 @@
       </c>
       <c r="W145" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:23)</t>
+          <t>Exceso de Jornada (01:44)</t>
         </is>
       </c>
     </row>
@@ -16939,12 +16975,12 @@
       </c>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>12:11</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:38</t>
         </is>
       </c>
       <c r="S147" s="7" t="inlineStr">
@@ -16954,7 +16990,7 @@
       </c>
       <c r="T147" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:38</t>
         </is>
       </c>
       <c r="U147" s="7" t="inlineStr">
@@ -16964,10 +17000,14 @@
       </c>
       <c r="V147" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W147" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W147" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:38)</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="5" t="inlineStr">
@@ -17052,7 +17092,7 @@
       </c>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
@@ -17621,7 +17661,7 @@
       </c>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
@@ -17960,12 +18000,12 @@
       </c>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="S156" s="7" t="inlineStr">
@@ -17975,7 +18015,7 @@
       </c>
       <c r="T156" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="U156" s="7" t="inlineStr">
@@ -17985,10 +18025,14 @@
       </c>
       <c r="V156" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W156" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W156" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:30)</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
@@ -18073,7 +18117,7 @@
       </c>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:26</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
@@ -18186,7 +18230,7 @@
       </c>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
@@ -18416,7 +18460,7 @@
       </c>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
@@ -18529,7 +18573,7 @@
       </c>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
@@ -18642,7 +18686,7 @@
       </c>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
@@ -18755,7 +18799,7 @@
       </c>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
@@ -18868,7 +18912,7 @@
       </c>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:18</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
@@ -19094,7 +19138,7 @@
       </c>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
@@ -19207,7 +19251,7 @@
       </c>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
@@ -19320,7 +19364,7 @@
       </c>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
@@ -19437,12 +19481,12 @@
       </c>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:37</t>
         </is>
       </c>
       <c r="S169" s="7" t="inlineStr">
@@ -19452,7 +19496,7 @@
       </c>
       <c r="T169" s="7" t="inlineStr">
         <is>
-          <t>02:00</t>
+          <t>02:37</t>
         </is>
       </c>
       <c r="U169" s="7" t="inlineStr">
@@ -19467,7 +19511,7 @@
       </c>
       <c r="W169" s="6" t="inlineStr">
         <is>
-          <t>Horas extras (02:00)</t>
+          <t>Horas extras (02:00), Exceso de Jornada (00:37)</t>
         </is>
       </c>
     </row>
@@ -19667,7 +19711,7 @@
       </c>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
@@ -19780,7 +19824,7 @@
       </c>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
@@ -19893,7 +19937,7 @@
       </c>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
@@ -20006,12 +20050,12 @@
       </c>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="S174" s="7" t="inlineStr">
@@ -20021,7 +20065,7 @@
       </c>
       <c r="T174" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:31</t>
         </is>
       </c>
       <c r="U174" s="7" t="inlineStr">
@@ -20031,10 +20075,14 @@
       </c>
       <c r="V174" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W174" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W174" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:31)</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="8" t="inlineStr">
@@ -20232,7 +20280,7 @@
       </c>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>12:01</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
@@ -20345,7 +20393,7 @@
       </c>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>10:29</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
@@ -20458,7 +20506,7 @@
       </c>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
@@ -20801,7 +20849,7 @@
       </c>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
@@ -20914,7 +20962,7 @@
       </c>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>10:02</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
@@ -21027,7 +21075,7 @@
       </c>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Revert "fix: Calculate worked hours and excess shift using real entry swipe timestamp instead of artificial snapping to 07:00/19:00"
This reverts commit 1c125fb2c0871da82cd9b7b695f35e058f455ffa.
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -866,7 +866,7 @@
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>12:26</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -979,12 +979,12 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:05</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>00:43</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>00:43</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
@@ -1004,14 +1004,10 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W7" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:43)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1322,7 +1318,7 @@
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
@@ -1435,12 +1431,12 @@
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S11" s="7" t="inlineStr">
@@ -1450,7 +1446,7 @@
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
@@ -1460,14 +1456,10 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W11" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:30)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -1782,7 +1774,7 @@
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
@@ -1895,7 +1887,7 @@
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
@@ -2008,7 +2000,7 @@
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>10:51</t>
+          <t>10:23</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
@@ -2121,12 +2113,12 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>14:09</t>
+          <t>13:56</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
         <is>
-          <t>02:09</t>
+          <t>01:56</t>
         </is>
       </c>
       <c r="S17" s="7" t="inlineStr">
@@ -2136,7 +2128,7 @@
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>02:09</t>
+          <t>01:56</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
@@ -2151,7 +2143,7 @@
       </c>
       <c r="W17" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (02:09)</t>
+          <t>Exceso de Jornada (01:56)</t>
         </is>
       </c>
     </row>
@@ -2238,12 +2230,12 @@
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S18" s="7" t="inlineStr">
@@ -2253,7 +2245,7 @@
       </c>
       <c r="T18" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U18" s="7" t="inlineStr">
@@ -2263,14 +2255,10 @@
       </c>
       <c r="V18" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W18" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:31)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W18" s="6" t="inlineStr"/>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -2355,7 +2343,7 @@
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
@@ -2468,7 +2456,7 @@
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:05</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
@@ -2694,7 +2682,7 @@
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
@@ -2924,7 +2912,7 @@
       </c>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
@@ -3037,7 +3025,7 @@
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>12:26</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
@@ -3150,7 +3138,7 @@
       </c>
       <c r="Q26" s="10" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="R26" s="10" t="inlineStr">
@@ -3384,12 +3372,12 @@
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>00:46</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S28" s="7" t="inlineStr">
@@ -3399,7 +3387,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>00:46</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
@@ -3409,12 +3397,12 @@
       </c>
       <c r="V28" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W28" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (00:46), Entrada duplicada (18:17)</t>
+          <t>Entrada duplicada (18:17)</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3489,7 @@
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>06:20</t>
+          <t>06:02</t>
         </is>
       </c>
       <c r="R29" s="7" t="inlineStr">
@@ -3531,7 +3519,7 @@
       </c>
       <c r="W29" s="6" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:20)</t>
+          <t>Jornada parcial (Medio día) (06:02)</t>
         </is>
       </c>
     </row>
@@ -3618,12 +3606,12 @@
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
         <is>
-          <t>00:34</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S30" s="7" t="inlineStr">
@@ -3633,7 +3621,7 @@
       </c>
       <c r="T30" s="7" t="inlineStr">
         <is>
-          <t>00:34</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U30" s="7" t="inlineStr">
@@ -3643,14 +3631,10 @@
       </c>
       <c r="V30" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W30" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:34)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W30" s="6" t="inlineStr"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
@@ -3735,7 +3719,7 @@
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
@@ -3848,7 +3832,7 @@
       </c>
       <c r="Q32" s="7" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R32" s="7" t="inlineStr">
@@ -3961,7 +3945,7 @@
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
@@ -4074,7 +4058,7 @@
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="R34" s="7" t="inlineStr">
@@ -4187,7 +4171,7 @@
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr">
@@ -4300,7 +4284,7 @@
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>12:16</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
@@ -4639,12 +4623,12 @@
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr">
         <is>
-          <t>00:34</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S39" s="7" t="inlineStr">
@@ -4654,7 +4638,7 @@
       </c>
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>04:34</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
@@ -4669,7 +4653,7 @@
       </c>
       <c r="W39" s="6" t="inlineStr">
         <is>
-          <t>Horas extras (04:00), Exceso de Jornada (00:34)</t>
+          <t>Horas extras (04:00)</t>
         </is>
       </c>
     </row>
@@ -4990,7 +4974,7 @@
       </c>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
@@ -5333,12 +5317,12 @@
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:12</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S45" s="7" t="inlineStr">
@@ -5348,7 +5332,7 @@
       </c>
       <c r="T45" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U45" s="7" t="inlineStr">
@@ -5358,14 +5342,10 @@
       </c>
       <c r="V45" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W45" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:30)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W45" s="6" t="inlineStr"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="5" t="inlineStr">
@@ -5450,7 +5430,7 @@
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
@@ -5676,12 +5656,12 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>00:56</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S48" s="7" t="inlineStr">
@@ -5691,7 +5671,7 @@
       </c>
       <c r="T48" s="7" t="inlineStr">
         <is>
-          <t>00:56</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U48" s="7" t="inlineStr">
@@ -5701,14 +5681,10 @@
       </c>
       <c r="V48" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W48" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:56)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W48" s="6" t="inlineStr"/>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -6136,12 +6112,12 @@
       </c>
       <c r="Q52" s="7" t="inlineStr">
         <is>
-          <t>12:44</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="R52" s="7" t="inlineStr">
         <is>
-          <t>00:44</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S52" s="7" t="inlineStr">
@@ -6151,7 +6127,7 @@
       </c>
       <c r="T52" s="7" t="inlineStr">
         <is>
-          <t>00:44</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U52" s="7" t="inlineStr">
@@ -6161,14 +6137,10 @@
       </c>
       <c r="V52" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W52" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:44)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W52" s="6" t="inlineStr"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="5" t="inlineStr">
@@ -6253,12 +6225,12 @@
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:09</t>
         </is>
       </c>
       <c r="R53" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S53" s="7" t="inlineStr">
@@ -6268,7 +6240,7 @@
       </c>
       <c r="T53" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U53" s="7" t="inlineStr">
@@ -6278,14 +6250,10 @@
       </c>
       <c r="V53" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W53" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:31)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W53" s="6" t="inlineStr"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
@@ -6483,12 +6451,12 @@
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="R55" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S55" s="7" t="inlineStr">
@@ -6498,7 +6466,7 @@
       </c>
       <c r="T55" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U55" s="7" t="inlineStr">
@@ -6508,14 +6476,10 @@
       </c>
       <c r="V55" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W55" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:31)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W55" s="6" t="inlineStr"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="5" t="inlineStr">
@@ -6713,7 +6677,7 @@
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
@@ -6826,7 +6790,7 @@
       </c>
       <c r="Q58" s="7" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="R58" s="7" t="inlineStr">
@@ -6939,12 +6903,12 @@
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>14:42</t>
         </is>
       </c>
       <c r="R59" s="7" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>02:42</t>
         </is>
       </c>
       <c r="S59" s="7" t="inlineStr">
@@ -6954,7 +6918,7 @@
       </c>
       <c r="T59" s="7" t="inlineStr">
         <is>
-          <t>03:02</t>
+          <t>02:42</t>
         </is>
       </c>
       <c r="U59" s="7" t="inlineStr">
@@ -6969,7 +6933,7 @@
       </c>
       <c r="W59" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (03:02), Entrada duplicada (06:40)</t>
+          <t>Exceso de Jornada (02:42), Entrada duplicada (06:40)</t>
         </is>
       </c>
     </row>
@@ -7056,7 +7020,7 @@
       </c>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
@@ -7173,12 +7137,12 @@
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="R61" s="7" t="inlineStr">
         <is>
-          <t>00:43</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="S61" s="7" t="inlineStr">
@@ -7188,7 +7152,7 @@
       </c>
       <c r="T61" s="7" t="inlineStr">
         <is>
-          <t>00:43</t>
+          <t>00:30</t>
         </is>
       </c>
       <c r="U61" s="7" t="inlineStr">
@@ -7203,7 +7167,7 @@
       </c>
       <c r="W61" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (00:43)</t>
+          <t>Exceso de Jornada (00:30)</t>
         </is>
       </c>
     </row>
@@ -8093,7 +8057,7 @@
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R69" s="7" t="inlineStr">
@@ -8206,7 +8170,7 @@
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
@@ -8319,7 +8283,7 @@
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
@@ -8545,7 +8509,7 @@
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>12:10</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R73" s="7" t="inlineStr">
@@ -8658,7 +8622,7 @@
       </c>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>10:20</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
@@ -8771,7 +8735,7 @@
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
@@ -9114,12 +9078,12 @@
       </c>
       <c r="Q78" s="7" t="inlineStr">
         <is>
-          <t>13:34</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="R78" s="7" t="inlineStr">
         <is>
-          <t>01:34</t>
+          <t>01:18</t>
         </is>
       </c>
       <c r="S78" s="7" t="inlineStr">
@@ -9129,7 +9093,7 @@
       </c>
       <c r="T78" s="7" t="inlineStr">
         <is>
-          <t>01:34</t>
+          <t>01:18</t>
         </is>
       </c>
       <c r="U78" s="7" t="inlineStr">
@@ -9144,7 +9108,7 @@
       </c>
       <c r="W78" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:34)</t>
+          <t>Exceso de Jornada (01:18)</t>
         </is>
       </c>
     </row>
@@ -9231,12 +9195,12 @@
       </c>
       <c r="Q79" s="7" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="R79" s="7" t="inlineStr">
         <is>
-          <t>02:59</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="S79" s="7" t="inlineStr">
@@ -9246,7 +9210,7 @@
       </c>
       <c r="T79" s="7" t="inlineStr">
         <is>
-          <t>02:59</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="U79" s="7" t="inlineStr">
@@ -9261,7 +9225,7 @@
       </c>
       <c r="W79" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (02:59)</t>
+          <t>Exceso de Jornada (02:38)</t>
         </is>
       </c>
     </row>
@@ -9348,7 +9312,7 @@
       </c>
       <c r="Q80" s="7" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R80" s="7" t="inlineStr">
@@ -9461,7 +9425,7 @@
       </c>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>12:16</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R81" s="7" t="inlineStr">
@@ -9687,7 +9651,7 @@
       </c>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R83" s="7" t="inlineStr">
@@ -9800,7 +9764,7 @@
       </c>
       <c r="Q84" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R84" s="7" t="inlineStr">
@@ -9913,7 +9877,7 @@
       </c>
       <c r="Q85" s="7" t="inlineStr">
         <is>
-          <t>12:16</t>
+          <t>12:06</t>
         </is>
       </c>
       <c r="R85" s="7" t="inlineStr">
@@ -10026,7 +9990,7 @@
       </c>
       <c r="Q86" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R86" s="7" t="inlineStr">
@@ -10256,7 +10220,7 @@
       </c>
       <c r="Q88" s="7" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R88" s="7" t="inlineStr">
@@ -10369,12 +10333,12 @@
       </c>
       <c r="Q89" s="7" t="inlineStr">
         <is>
-          <t>13:29</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="R89" s="7" t="inlineStr">
         <is>
-          <t>01:29</t>
+          <t>01:17</t>
         </is>
       </c>
       <c r="S89" s="7" t="inlineStr">
@@ -10384,7 +10348,7 @@
       </c>
       <c r="T89" s="7" t="inlineStr">
         <is>
-          <t>01:29</t>
+          <t>01:17</t>
         </is>
       </c>
       <c r="U89" s="7" t="inlineStr">
@@ -10399,7 +10363,7 @@
       </c>
       <c r="W89" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:29)</t>
+          <t>Exceso de Jornada (01:17)</t>
         </is>
       </c>
     </row>
@@ -10486,12 +10450,12 @@
       </c>
       <c r="Q90" s="7" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="R90" s="7" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="S90" s="7" t="inlineStr">
@@ -10501,7 +10465,7 @@
       </c>
       <c r="T90" s="7" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>02:38</t>
         </is>
       </c>
       <c r="U90" s="7" t="inlineStr">
@@ -10516,7 +10480,7 @@
       </c>
       <c r="W90" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (02:56)</t>
+          <t>Exceso de Jornada (02:38)</t>
         </is>
       </c>
     </row>
@@ -10603,7 +10567,7 @@
       </c>
       <c r="Q91" s="7" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R91" s="7" t="inlineStr">
@@ -10716,7 +10680,7 @@
       </c>
       <c r="Q92" s="7" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R92" s="7" t="inlineStr">
@@ -11059,7 +11023,7 @@
       </c>
       <c r="Q95" s="7" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="R95" s="7" t="inlineStr">
@@ -11172,7 +11136,7 @@
       </c>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
@@ -11858,7 +11822,7 @@
       </c>
       <c r="Q102" s="7" t="inlineStr">
         <is>
-          <t>12:16</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R102" s="7" t="inlineStr">
@@ -12197,7 +12161,7 @@
       </c>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>06:07</t>
+          <t>05:55</t>
         </is>
       </c>
       <c r="R105" s="7" t="inlineStr">
@@ -12227,7 +12191,7 @@
       </c>
       <c r="W105" s="6" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:07)</t>
+          <t>Jornada parcial (Medio día) (05:55)</t>
         </is>
       </c>
     </row>
@@ -12314,7 +12278,7 @@
       </c>
       <c r="Q106" s="7" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R106" s="7" t="inlineStr">
@@ -12427,7 +12391,7 @@
       </c>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="R107" s="7" t="inlineStr">
@@ -12540,7 +12504,7 @@
       </c>
       <c r="Q108" s="7" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R108" s="7" t="inlineStr">
@@ -12766,7 +12730,7 @@
       </c>
       <c r="Q110" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="R110" s="7" t="inlineStr">
@@ -12879,7 +12843,7 @@
       </c>
       <c r="Q111" s="7" t="inlineStr">
         <is>
-          <t>12:16</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R111" s="7" t="inlineStr">
@@ -12992,7 +12956,7 @@
       </c>
       <c r="Q112" s="7" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="R112" s="7" t="inlineStr">
@@ -13218,7 +13182,7 @@
       </c>
       <c r="Q114" s="7" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R114" s="7" t="inlineStr">
@@ -13331,7 +13295,7 @@
       </c>
       <c r="Q115" s="7" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="R115" s="7" t="inlineStr">
@@ -13444,7 +13408,7 @@
       </c>
       <c r="Q116" s="7" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="R116" s="7" t="inlineStr">
@@ -13787,7 +13751,7 @@
       </c>
       <c r="Q119" s="7" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="R119" s="7" t="inlineStr">
@@ -13900,7 +13864,7 @@
       </c>
       <c r="Q120" s="7" t="inlineStr">
         <is>
-          <t>10:31</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="R120" s="7" t="inlineStr">
@@ -14013,7 +13977,7 @@
       </c>
       <c r="Q121" s="7" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="R121" s="7" t="inlineStr">
@@ -14126,7 +14090,7 @@
       </c>
       <c r="Q122" s="7" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>11:59</t>
         </is>
       </c>
       <c r="R122" s="7" t="inlineStr">
@@ -14352,7 +14316,7 @@
       </c>
       <c r="Q124" s="7" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="R124" s="7" t="inlineStr">
@@ -14465,7 +14429,7 @@
       </c>
       <c r="Q125" s="7" t="inlineStr">
         <is>
-          <t>10:22</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="R125" s="7" t="inlineStr">
@@ -14925,7 +14889,7 @@
       </c>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:13</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
@@ -15151,7 +15115,7 @@
       </c>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -15264,7 +15228,7 @@
       </c>
       <c r="Q132" s="7" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R132" s="7" t="inlineStr">
@@ -15377,7 +15341,7 @@
       </c>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
@@ -15490,7 +15454,7 @@
       </c>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
@@ -15518,7 +15482,11 @@
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="W134" s="6" t="inlineStr"/>
+      <c r="W134" s="6" t="inlineStr">
+        <is>
+          <t>Jornada parcial (Medio día) (07:55)</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
@@ -15603,7 +15571,7 @@
       </c>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>06:18</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
@@ -15633,7 +15601,7 @@
       </c>
       <c r="W135" s="6" t="inlineStr">
         <is>
-          <t>Jornada parcial (Medio día) (06:18)</t>
+          <t>Jornada parcial (Medio día) (06:00)</t>
         </is>
       </c>
     </row>
@@ -15720,7 +15688,7 @@
       </c>
       <c r="Q136" s="7" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R136" s="7" t="inlineStr">
@@ -15833,7 +15801,7 @@
       </c>
       <c r="Q137" s="7" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="R137" s="7" t="inlineStr">
@@ -15946,7 +15914,7 @@
       </c>
       <c r="Q138" s="7" t="inlineStr">
         <is>
-          <t>12:13</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R138" s="7" t="inlineStr">
@@ -16059,7 +16027,7 @@
       </c>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>11:59</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
@@ -16172,12 +16140,12 @@
       </c>
       <c r="Q140" s="7" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R140" s="7" t="inlineStr">
         <is>
-          <t>00:32</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S140" s="7" t="inlineStr">
@@ -16187,7 +16155,7 @@
       </c>
       <c r="T140" s="7" t="inlineStr">
         <is>
-          <t>00:32</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U140" s="7" t="inlineStr">
@@ -16197,14 +16165,10 @@
       </c>
       <c r="V140" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W140" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:32)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W140" s="6" t="inlineStr"/>
     </row>
     <row r="141" ht="20" customHeight="1">
       <c r="A141" s="5" t="inlineStr">
@@ -16289,7 +16253,7 @@
       </c>
       <c r="Q141" s="7" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="R141" s="7" t="inlineStr">
@@ -16402,7 +16366,7 @@
       </c>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
@@ -16628,12 +16592,12 @@
       </c>
       <c r="Q144" s="7" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R144" s="7" t="inlineStr">
         <is>
-          <t>00:38</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S144" s="7" t="inlineStr">
@@ -16643,7 +16607,7 @@
       </c>
       <c r="T144" s="7" t="inlineStr">
         <is>
-          <t>00:38</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U144" s="7" t="inlineStr">
@@ -16653,12 +16617,12 @@
       </c>
       <c r="V144" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W144" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (00:38), Entrada duplicada (06:36, 06:37)</t>
+          <t>Entrada duplicada (06:36, 06:37)</t>
         </is>
       </c>
     </row>
@@ -16745,12 +16709,12 @@
       </c>
       <c r="Q145" s="7" t="inlineStr">
         <is>
-          <t>13:44</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="R145" s="7" t="inlineStr">
         <is>
-          <t>01:44</t>
+          <t>01:23</t>
         </is>
       </c>
       <c r="S145" s="7" t="inlineStr">
@@ -16760,7 +16724,7 @@
       </c>
       <c r="T145" s="7" t="inlineStr">
         <is>
-          <t>01:44</t>
+          <t>01:23</t>
         </is>
       </c>
       <c r="U145" s="7" t="inlineStr">
@@ -16775,7 +16739,7 @@
       </c>
       <c r="W145" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (01:44)</t>
+          <t>Exceso de Jornada (01:23)</t>
         </is>
       </c>
     </row>
@@ -16975,12 +16939,12 @@
       </c>
       <c r="Q147" s="7" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:11</t>
         </is>
       </c>
       <c r="R147" s="7" t="inlineStr">
         <is>
-          <t>00:38</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S147" s="7" t="inlineStr">
@@ -16990,7 +16954,7 @@
       </c>
       <c r="T147" s="7" t="inlineStr">
         <is>
-          <t>00:38</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U147" s="7" t="inlineStr">
@@ -17000,14 +16964,10 @@
       </c>
       <c r="V147" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W147" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:38)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W147" s="6" t="inlineStr"/>
     </row>
     <row r="148" ht="20" customHeight="1">
       <c r="A148" s="5" t="inlineStr">
@@ -17092,7 +17052,7 @@
       </c>
       <c r="Q148" s="7" t="inlineStr">
         <is>
-          <t>12:20</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R148" s="7" t="inlineStr">
@@ -17661,7 +17621,7 @@
       </c>
       <c r="Q153" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="R153" s="7" t="inlineStr">
@@ -18000,12 +17960,12 @@
       </c>
       <c r="Q156" s="7" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="R156" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S156" s="7" t="inlineStr">
@@ -18015,7 +17975,7 @@
       </c>
       <c r="T156" s="7" t="inlineStr">
         <is>
-          <t>00:30</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U156" s="7" t="inlineStr">
@@ -18025,14 +17985,10 @@
       </c>
       <c r="V156" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W156" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:30)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W156" s="6" t="inlineStr"/>
     </row>
     <row r="157" ht="20" customHeight="1">
       <c r="A157" s="5" t="inlineStr">
@@ -18117,7 +18073,7 @@
       </c>
       <c r="Q157" s="7" t="inlineStr">
         <is>
-          <t>12:26</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="R157" s="7" t="inlineStr">
@@ -18230,7 +18186,7 @@
       </c>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
@@ -18460,7 +18416,7 @@
       </c>
       <c r="Q160" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="R160" s="7" t="inlineStr">
@@ -18573,7 +18529,7 @@
       </c>
       <c r="Q161" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R161" s="7" t="inlineStr">
@@ -18686,7 +18642,7 @@
       </c>
       <c r="Q162" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="R162" s="7" t="inlineStr">
@@ -18799,7 +18755,7 @@
       </c>
       <c r="Q163" s="7" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="R163" s="7" t="inlineStr">
@@ -18912,7 +18868,7 @@
       </c>
       <c r="Q164" s="7" t="inlineStr">
         <is>
-          <t>12:18</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="R164" s="7" t="inlineStr">
@@ -19138,7 +19094,7 @@
       </c>
       <c r="Q166" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="R166" s="7" t="inlineStr">
@@ -19251,7 +19207,7 @@
       </c>
       <c r="Q167" s="7" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="R167" s="7" t="inlineStr">
@@ -19364,7 +19320,7 @@
       </c>
       <c r="Q168" s="7" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="R168" s="7" t="inlineStr">
@@ -19481,12 +19437,12 @@
       </c>
       <c r="Q169" s="7" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:14</t>
         </is>
       </c>
       <c r="R169" s="7" t="inlineStr">
         <is>
-          <t>00:37</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S169" s="7" t="inlineStr">
@@ -19496,7 +19452,7 @@
       </c>
       <c r="T169" s="7" t="inlineStr">
         <is>
-          <t>02:37</t>
+          <t>02:00</t>
         </is>
       </c>
       <c r="U169" s="7" t="inlineStr">
@@ -19511,7 +19467,7 @@
       </c>
       <c r="W169" s="6" t="inlineStr">
         <is>
-          <t>Horas extras (02:00), Exceso de Jornada (00:37)</t>
+          <t>Horas extras (02:00)</t>
         </is>
       </c>
     </row>
@@ -19711,7 +19667,7 @@
       </c>
       <c r="Q171" s="7" t="inlineStr">
         <is>
-          <t>12:14</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R171" s="7" t="inlineStr">
@@ -19824,7 +19780,7 @@
       </c>
       <c r="Q172" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R172" s="7" t="inlineStr">
@@ -19937,7 +19893,7 @@
       </c>
       <c r="Q173" s="7" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R173" s="7" t="inlineStr">
@@ -20050,12 +20006,12 @@
       </c>
       <c r="Q174" s="7" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="R174" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S174" s="7" t="inlineStr">
@@ -20065,7 +20021,7 @@
       </c>
       <c r="T174" s="7" t="inlineStr">
         <is>
-          <t>00:31</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U174" s="7" t="inlineStr">
@@ -20075,14 +20031,10 @@
       </c>
       <c r="V174" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W174" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:31)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W174" s="6" t="inlineStr"/>
     </row>
     <row r="175" ht="20" customHeight="1">
       <c r="A175" s="8" t="inlineStr">
@@ -20280,7 +20232,7 @@
       </c>
       <c r="Q176" s="7" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="R176" s="7" t="inlineStr">
@@ -20393,7 +20345,7 @@
       </c>
       <c r="Q177" s="7" t="inlineStr">
         <is>
-          <t>10:29</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="R177" s="7" t="inlineStr">
@@ -20506,7 +20458,7 @@
       </c>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
@@ -20849,7 +20801,7 @@
       </c>
       <c r="Q181" s="7" t="inlineStr">
         <is>
-          <t>12:29</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R181" s="7" t="inlineStr">
@@ -20962,7 +20914,7 @@
       </c>
       <c r="Q182" s="7" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="R182" s="7" t="inlineStr">
@@ -21075,7 +21027,7 @@
       </c>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat: Implemented Mantenimiento rule with 06:25 AM cut-off threshold for real entry swipe worked hours calculation
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -979,12 +979,12 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>12:05</t>
+          <t>12:43</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:43</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:43</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
@@ -1004,10 +1004,14 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W7" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:43)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -3372,12 +3376,12 @@
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>12:02</t>
+          <t>12:46</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:46</t>
         </is>
       </c>
       <c r="S28" s="7" t="inlineStr">
@@ -3387,7 +3391,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:46</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
@@ -3397,12 +3401,12 @@
       </c>
       <c r="V28" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Exceso de Jornada</t>
         </is>
       </c>
       <c r="W28" s="6" t="inlineStr">
         <is>
-          <t>Entrada duplicada (18:17)</t>
+          <t>Exceso de Jornada (00:46), Entrada duplicada (18:17)</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3949,7 @@
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>12:07</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
@@ -5430,7 +5434,7 @@
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
@@ -5656,12 +5660,12 @@
       </c>
       <c r="Q48" s="7" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="R48" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:56</t>
         </is>
       </c>
       <c r="S48" s="7" t="inlineStr">
@@ -5671,7 +5675,7 @@
       </c>
       <c r="T48" s="7" t="inlineStr">
         <is>
-          <t>00:00</t>
+          <t>00:56</t>
         </is>
       </c>
       <c r="U48" s="7" t="inlineStr">
@@ -5681,10 +5685,14 @@
       </c>
       <c r="V48" s="7" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="W48" s="6" t="inlineStr"/>
+          <t>Exceso de Jornada</t>
+        </is>
+      </c>
+      <c r="W48" s="6" t="inlineStr">
+        <is>
+          <t>Exceso de Jornada (00:56)</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -6677,7 +6685,7 @@
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
@@ -8735,7 +8743,7 @@
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
@@ -11136,7 +11144,7 @@
       </c>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
@@ -13408,7 +13416,7 @@
       </c>
       <c r="Q116" s="7" t="inlineStr">
         <is>
-          <t>14:01</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="R116" s="7" t="inlineStr">
@@ -13977,7 +13985,7 @@
       </c>
       <c r="Q121" s="7" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="R121" s="7" t="inlineStr">
@@ -15115,7 +15123,7 @@
       </c>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -15454,7 +15462,7 @@
       </c>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
@@ -15482,11 +15490,7 @@
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="W134" s="6" t="inlineStr">
-        <is>
-          <t>Jornada parcial (Medio día) (07:55)</t>
-        </is>
-      </c>
+      <c r="W134" s="6" t="inlineStr"/>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
@@ -16027,7 +16031,7 @@
       </c>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:59</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
@@ -16366,7 +16370,7 @@
       </c>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
@@ -18186,7 +18190,7 @@
       </c>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
@@ -20458,7 +20462,7 @@
       </c>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
@@ -21027,7 +21031,7 @@
       </c>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>14:05</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">

</xml_diff>

<commit_message>
fix: Restrict Mantenimiento rule to strictly match Posición/Cargo == Mantenimiento (ignoring department/Oper&Mtto)
</commit_message>
<xml_diff>
--- a/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
+++ b/Reporte_Asistencia_GZG_2026-08-17_al_2026-08-21.xlsx
@@ -979,12 +979,12 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>12:43</t>
+          <t>12:05</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
         <is>
-          <t>00:43</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S7" s="7" t="inlineStr">
@@ -994,7 +994,7 @@
       </c>
       <c r="T7" s="7" t="inlineStr">
         <is>
-          <t>00:43</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U7" s="7" t="inlineStr">
@@ -1004,14 +1004,10 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
-        </is>
-      </c>
-      <c r="W7" s="6" t="inlineStr">
-        <is>
-          <t>Exceso de Jornada (00:43)</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="W7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -3376,12 +3372,12 @@
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>12:46</t>
+          <t>12:02</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
         <is>
-          <t>00:46</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="S28" s="7" t="inlineStr">
@@ -3391,7 +3387,7 @@
       </c>
       <c r="T28" s="7" t="inlineStr">
         <is>
-          <t>00:46</t>
+          <t>00:00</t>
         </is>
       </c>
       <c r="U28" s="7" t="inlineStr">
@@ -3401,12 +3397,12 @@
       </c>
       <c r="V28" s="7" t="inlineStr">
         <is>
-          <t>Exceso de Jornada</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="W28" s="6" t="inlineStr">
         <is>
-          <t>Exceso de Jornada (00:46), Entrada duplicada (18:17)</t>
+          <t>Entrada duplicada (18:17)</t>
         </is>
       </c>
     </row>
@@ -3949,7 +3945,7 @@
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>12:07</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
@@ -5434,7 +5430,7 @@
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
@@ -6685,7 +6681,7 @@
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
@@ -8743,7 +8739,7 @@
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>14:20</t>
+          <t>14:10</t>
         </is>
       </c>
       <c r="R75" s="7" t="inlineStr">
@@ -11144,7 +11140,7 @@
       </c>
       <c r="Q96" s="7" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="R96" s="7" t="inlineStr">
@@ -13416,7 +13412,7 @@
       </c>
       <c r="Q116" s="7" t="inlineStr">
         <is>
-          <t>14:04</t>
+          <t>14:01</t>
         </is>
       </c>
       <c r="R116" s="7" t="inlineStr">
@@ -13985,7 +13981,7 @@
       </c>
       <c r="Q121" s="7" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="R121" s="7" t="inlineStr">
@@ -15123,7 +15119,7 @@
       </c>
       <c r="Q131" s="7" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R131" s="7" t="inlineStr">
@@ -15462,7 +15458,7 @@
       </c>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>08:01</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
@@ -15490,7 +15486,11 @@
           <t>Cambio de guardia</t>
         </is>
       </c>
-      <c r="W134" s="6" t="inlineStr"/>
+      <c r="W134" s="6" t="inlineStr">
+        <is>
+          <t>Jornada parcial (Medio día) (07:55)</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="20" customHeight="1">
       <c r="A135" s="5" t="inlineStr">
@@ -16031,7 +16031,7 @@
       </c>
       <c r="Q139" s="7" t="inlineStr">
         <is>
-          <t>11:59</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R139" s="7" t="inlineStr">
@@ -16370,7 +16370,7 @@
       </c>
       <c r="Q142" s="7" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="R142" s="7" t="inlineStr">
@@ -18190,7 +18190,7 @@
       </c>
       <c r="Q158" s="7" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="R158" s="7" t="inlineStr">
@@ -20462,7 +20462,7 @@
       </c>
       <c r="Q178" s="7" t="inlineStr">
         <is>
-          <t>14:10</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="R178" s="7" t="inlineStr">
@@ -21031,7 +21031,7 @@
       </c>
       <c r="Q183" s="7" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:05</t>
         </is>
       </c>
       <c r="R183" s="7" t="inlineStr">

</xml_diff>